<commit_message>
Teklif dökümantasyonu v2: 5 firma fiyatları + döviz formatı
Yeni firmalar: AYVAZ (TL/USD), CENKSAN (TL), KLINGER (EUR)
Güncelleme: Compact firma ataması (boşluksuz sıralama)
Döviz formatı: ₺ TL, $ USD, € EUR hücre formatı olarak eklendi
Eşleşen 22 OZEL kalemi dolduruldu
</commit_message>
<xml_diff>
--- a/TEKLIF DOKUMANTASYON.xlsx
+++ b/TEKLIF DOKUMANTASYON.xlsx
@@ -20,9 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="000"/>
     <numFmt numFmtId="165" formatCode="_-[$₺-41F]* #,##0.00_-;\-[$₺-41F]* #,##0.00_-;_-[$₺-41F]* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="&quot;€&quot;#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="₺#,##0.00"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -382,7 +385,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -600,7 +603,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -612,7 +615,16 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5016,7 +5028,9 @@
       </c>
       <c r="E62" s="60" t="n"/>
       <c r="F62" s="60" t="n"/>
-      <c r="G62" s="91" t="n"/>
+      <c r="G62" s="96" t="n">
+        <v>1315</v>
+      </c>
       <c r="H62" s="91" t="n"/>
       <c r="I62" s="91" t="n"/>
       <c r="J62" s="91" t="n"/>
@@ -5025,7 +5039,11 @@
         <f>IFERROR(AVERAGEIF(G62:K62,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M62" s="93" t="n"/>
+      <c r="M62" s="93" t="inlineStr">
+        <is>
+          <t>KLINGER</t>
+        </is>
+      </c>
       <c r="N62" s="93" t="n"/>
       <c r="O62" s="93" t="n"/>
       <c r="P62" s="93" t="n"/>
@@ -5060,7 +5078,9 @@
       </c>
       <c r="E63" s="60" t="n"/>
       <c r="F63" s="60" t="n"/>
-      <c r="G63" s="91" t="n"/>
+      <c r="G63" s="96" t="n">
+        <v>300</v>
+      </c>
       <c r="H63" s="91" t="n"/>
       <c r="I63" s="91" t="n"/>
       <c r="J63" s="91" t="n"/>
@@ -5069,7 +5089,11 @@
         <f>IFERROR(AVERAGEIF(G63:K63,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M63" s="93" t="n"/>
+      <c r="M63" s="93" t="inlineStr">
+        <is>
+          <t>KLINGER</t>
+        </is>
+      </c>
       <c r="N63" s="93" t="n"/>
       <c r="O63" s="93" t="n"/>
       <c r="P63" s="93" t="n"/>
@@ -5236,7 +5260,9 @@
       </c>
       <c r="E67" s="60" t="n"/>
       <c r="F67" s="60" t="n"/>
-      <c r="G67" s="91" t="n"/>
+      <c r="G67" s="96" t="n">
+        <v>370</v>
+      </c>
       <c r="H67" s="91" t="n"/>
       <c r="I67" s="91" t="n"/>
       <c r="J67" s="91" t="n"/>
@@ -5245,7 +5271,11 @@
         <f>IFERROR(AVERAGEIF(G67:K67,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M67" s="93" t="n"/>
+      <c r="M67" s="93" t="inlineStr">
+        <is>
+          <t>KLINGER</t>
+        </is>
+      </c>
       <c r="N67" s="93" t="n"/>
       <c r="O67" s="93" t="n"/>
       <c r="P67" s="93" t="n"/>
@@ -5368,7 +5398,9 @@
       </c>
       <c r="E70" s="60" t="n"/>
       <c r="F70" s="60" t="n"/>
-      <c r="G70" s="91" t="n"/>
+      <c r="G70" s="96" t="n">
+        <v>525</v>
+      </c>
       <c r="H70" s="91" t="n"/>
       <c r="I70" s="91" t="n"/>
       <c r="J70" s="91" t="n"/>
@@ -5377,7 +5409,11 @@
         <f>IFERROR(AVERAGEIF(G70:K70,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M70" s="93" t="n"/>
+      <c r="M70" s="93" t="inlineStr">
+        <is>
+          <t>KLINGER</t>
+        </is>
+      </c>
       <c r="N70" s="93" t="n"/>
       <c r="O70" s="93" t="n"/>
       <c r="P70" s="93" t="n"/>
@@ -8801,10 +8837,10 @@
       </c>
       <c r="E148" s="60" t="n"/>
       <c r="F148" s="60" t="n"/>
-      <c r="G148" s="91" t="n">
+      <c r="G148" s="96" t="n">
         <v>73.34999999999999</v>
       </c>
-      <c r="H148" s="91" t="n">
+      <c r="H148" s="97" t="n">
         <v>65.48999999999999</v>
       </c>
       <c r="I148" s="91" t="n"/>
@@ -8857,10 +8893,10 @@
       </c>
       <c r="E149" s="60" t="n"/>
       <c r="F149" s="60" t="n"/>
-      <c r="G149" s="91" t="n">
+      <c r="G149" s="96" t="n">
         <v>31.8</v>
       </c>
-      <c r="H149" s="91" t="n">
+      <c r="H149" s="97" t="n">
         <v>35.28</v>
       </c>
       <c r="I149" s="91" t="n"/>
@@ -8913,10 +8949,10 @@
       </c>
       <c r="E150" s="60" t="n"/>
       <c r="F150" s="60" t="n"/>
-      <c r="G150" s="91" t="n">
+      <c r="G150" s="96" t="n">
         <v>28.55</v>
       </c>
-      <c r="H150" s="91" t="n">
+      <c r="H150" s="97" t="n">
         <v>35.28</v>
       </c>
       <c r="I150" s="91" t="n"/>
@@ -8969,10 +9005,10 @@
       </c>
       <c r="E151" s="60" t="n"/>
       <c r="F151" s="60" t="n"/>
-      <c r="G151" s="91" t="n">
+      <c r="G151" s="96" t="n">
         <v>37.5</v>
       </c>
-      <c r="H151" s="91" t="n">
+      <c r="H151" s="97" t="n">
         <v>45.9</v>
       </c>
       <c r="I151" s="91" t="n"/>
@@ -9025,10 +9061,10 @@
       </c>
       <c r="E152" s="60" t="n"/>
       <c r="F152" s="60" t="n"/>
-      <c r="G152" s="91" t="n">
+      <c r="G152" s="96" t="n">
         <v>47.9</v>
       </c>
-      <c r="H152" s="91" t="n">
+      <c r="H152" s="97" t="n">
         <v>45.9</v>
       </c>
       <c r="I152" s="91" t="n"/>
@@ -9081,10 +9117,10 @@
       </c>
       <c r="E153" s="60" t="n"/>
       <c r="F153" s="60" t="n"/>
-      <c r="G153" s="91" t="n">
+      <c r="G153" s="96" t="n">
         <v>336.25</v>
       </c>
-      <c r="H153" s="91" t="n">
+      <c r="H153" s="97" t="n">
         <v>362.61</v>
       </c>
       <c r="I153" s="91" t="n"/>
@@ -9137,10 +9173,10 @@
       </c>
       <c r="E154" s="60" t="n"/>
       <c r="F154" s="60" t="n"/>
-      <c r="G154" s="91" t="n"/>
-      <c r="H154" s="91" t="n">
+      <c r="G154" s="97" t="n">
         <v>98.33</v>
       </c>
+      <c r="H154" s="91" t="n"/>
       <c r="I154" s="91" t="n"/>
       <c r="J154" s="91" t="n"/>
       <c r="K154" s="91" t="n"/>
@@ -9148,12 +9184,12 @@
         <f>IFERROR(AVERAGEIF(G154:K154,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M154" s="93" t="n"/>
-      <c r="N154" s="93" t="inlineStr">
+      <c r="M154" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N154" s="93" t="n"/>
       <c r="O154" s="93" t="n"/>
       <c r="P154" s="93" t="n"/>
       <c r="Q154" s="93" t="n"/>
@@ -9187,10 +9223,10 @@
       </c>
       <c r="E155" s="60" t="n"/>
       <c r="F155" s="60" t="n"/>
-      <c r="G155" s="91" t="n"/>
-      <c r="H155" s="91" t="n">
+      <c r="G155" s="97" t="n">
         <v>216.33</v>
       </c>
+      <c r="H155" s="91" t="n"/>
       <c r="I155" s="91" t="n"/>
       <c r="J155" s="91" t="n"/>
       <c r="K155" s="91" t="n"/>
@@ -9198,12 +9234,12 @@
         <f>IFERROR(AVERAGEIF(G155:K155,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M155" s="93" t="n"/>
-      <c r="N155" s="93" t="inlineStr">
+      <c r="M155" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N155" s="93" t="n"/>
       <c r="O155" s="93" t="n"/>
       <c r="P155" s="93" t="n"/>
       <c r="Q155" s="93" t="n"/>
@@ -9237,10 +9273,10 @@
       </c>
       <c r="E156" s="60" t="n"/>
       <c r="F156" s="60" t="n"/>
-      <c r="G156" s="91" t="n"/>
-      <c r="H156" s="91" t="n">
+      <c r="G156" s="97" t="n">
         <v>20.06</v>
       </c>
+      <c r="H156" s="91" t="n"/>
       <c r="I156" s="91" t="n"/>
       <c r="J156" s="91" t="n"/>
       <c r="K156" s="91" t="n"/>
@@ -9248,12 +9284,12 @@
         <f>IFERROR(AVERAGEIF(G156:K156,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M156" s="93" t="n"/>
-      <c r="N156" s="93" t="inlineStr">
+      <c r="M156" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N156" s="93" t="n"/>
       <c r="O156" s="93" t="n"/>
       <c r="P156" s="93" t="n"/>
       <c r="Q156" s="93" t="n"/>
@@ -9287,10 +9323,10 @@
       </c>
       <c r="E157" s="60" t="n"/>
       <c r="F157" s="60" t="n"/>
-      <c r="G157" s="91" t="n"/>
-      <c r="H157" s="91" t="n">
+      <c r="G157" s="97" t="n">
         <v>41.96</v>
       </c>
+      <c r="H157" s="91" t="n"/>
       <c r="I157" s="91" t="n"/>
       <c r="J157" s="91" t="n"/>
       <c r="K157" s="91" t="n"/>
@@ -9298,12 +9334,12 @@
         <f>IFERROR(AVERAGEIF(G157:K157,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M157" s="93" t="n"/>
-      <c r="N157" s="93" t="inlineStr">
+      <c r="M157" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N157" s="93" t="n"/>
       <c r="O157" s="93" t="n"/>
       <c r="P157" s="93" t="n"/>
       <c r="Q157" s="93" t="n"/>
@@ -9337,10 +9373,10 @@
       </c>
       <c r="E158" s="60" t="n"/>
       <c r="F158" s="60" t="n"/>
-      <c r="G158" s="91" t="n"/>
-      <c r="H158" s="91" t="n">
+      <c r="G158" s="97" t="n">
         <v>285.82</v>
       </c>
+      <c r="H158" s="91" t="n"/>
       <c r="I158" s="91" t="n"/>
       <c r="J158" s="91" t="n"/>
       <c r="K158" s="91" t="n"/>
@@ -9348,12 +9384,12 @@
         <f>IFERROR(AVERAGEIF(G158:K158,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M158" s="93" t="n"/>
-      <c r="N158" s="93" t="inlineStr">
+      <c r="M158" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N158" s="93" t="n"/>
       <c r="O158" s="93" t="n"/>
       <c r="P158" s="93" t="n"/>
       <c r="Q158" s="93" t="n"/>
@@ -9387,10 +9423,10 @@
       </c>
       <c r="E159" s="60" t="n"/>
       <c r="F159" s="60" t="n"/>
-      <c r="G159" s="91" t="n"/>
-      <c r="H159" s="91" t="n">
+      <c r="G159" s="97" t="n">
         <v>26.22</v>
       </c>
+      <c r="H159" s="91" t="n"/>
       <c r="I159" s="91" t="n"/>
       <c r="J159" s="91" t="n"/>
       <c r="K159" s="91" t="n"/>
@@ -9398,12 +9434,12 @@
         <f>IFERROR(AVERAGEIF(G159:K159,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M159" s="93" t="n"/>
-      <c r="N159" s="93" t="inlineStr">
+      <c r="M159" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N159" s="93" t="n"/>
       <c r="O159" s="93" t="n"/>
       <c r="P159" s="93" t="n"/>
       <c r="Q159" s="93" t="n"/>
@@ -9437,10 +9473,10 @@
       </c>
       <c r="E160" s="60" t="n"/>
       <c r="F160" s="60" t="n"/>
-      <c r="G160" s="91" t="n"/>
-      <c r="H160" s="91" t="n">
+      <c r="G160" s="97" t="n">
         <v>56.38</v>
       </c>
+      <c r="H160" s="91" t="n"/>
       <c r="I160" s="91" t="n"/>
       <c r="J160" s="91" t="n"/>
       <c r="K160" s="91" t="n"/>
@@ -9448,12 +9484,12 @@
         <f>IFERROR(AVERAGEIF(G160:K160,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M160" s="93" t="n"/>
-      <c r="N160" s="93" t="inlineStr">
+      <c r="M160" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N160" s="93" t="n"/>
       <c r="O160" s="93" t="n"/>
       <c r="P160" s="93" t="n"/>
       <c r="Q160" s="93" t="n"/>
@@ -9487,10 +9523,10 @@
       </c>
       <c r="E161" s="60" t="n"/>
       <c r="F161" s="60" t="n"/>
-      <c r="G161" s="91" t="n"/>
-      <c r="H161" s="91" t="n">
+      <c r="G161" s="97" t="n">
         <v>2.49</v>
       </c>
+      <c r="H161" s="91" t="n"/>
       <c r="I161" s="91" t="n"/>
       <c r="J161" s="91" t="n"/>
       <c r="K161" s="91" t="n"/>
@@ -9498,12 +9534,12 @@
         <f>IFERROR(AVERAGEIF(G161:K161,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M161" s="93" t="n"/>
-      <c r="N161" s="93" t="inlineStr">
+      <c r="M161" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N161" s="93" t="n"/>
       <c r="O161" s="93" t="n"/>
       <c r="P161" s="93" t="n"/>
       <c r="Q161" s="93" t="n"/>
@@ -9537,10 +9573,10 @@
       </c>
       <c r="E162" s="60" t="n"/>
       <c r="F162" s="60" t="n"/>
-      <c r="G162" s="91" t="n"/>
-      <c r="H162" s="91" t="n">
+      <c r="G162" s="97" t="n">
         <v>3.8</v>
       </c>
+      <c r="H162" s="91" t="n"/>
       <c r="I162" s="91" t="n"/>
       <c r="J162" s="91" t="n"/>
       <c r="K162" s="91" t="n"/>
@@ -9548,12 +9584,12 @@
         <f>IFERROR(AVERAGEIF(G162:K162,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M162" s="93" t="n"/>
-      <c r="N162" s="93" t="inlineStr">
+      <c r="M162" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N162" s="93" t="n"/>
       <c r="O162" s="93" t="n"/>
       <c r="P162" s="93" t="n"/>
       <c r="Q162" s="93" t="n"/>
@@ -9588,10 +9624,10 @@
       </c>
       <c r="E163" s="60" t="n"/>
       <c r="F163" s="60" t="n"/>
-      <c r="G163" s="91" t="n"/>
-      <c r="H163" s="91" t="n">
+      <c r="G163" s="97" t="n">
         <v>10.36</v>
       </c>
+      <c r="H163" s="91" t="n"/>
       <c r="I163" s="91" t="n"/>
       <c r="J163" s="91" t="n"/>
       <c r="K163" s="91" t="n"/>
@@ -9599,12 +9635,12 @@
         <f>IFERROR(AVERAGEIF(G163:K163,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M163" s="93" t="n"/>
-      <c r="N163" s="93" t="inlineStr">
+      <c r="M163" s="93" t="inlineStr">
         <is>
           <t>HERA ÇELİK</t>
         </is>
       </c>
+      <c r="N163" s="93" t="n"/>
       <c r="O163" s="93" t="n"/>
       <c r="P163" s="93" t="n"/>
       <c r="Q163" s="93" t="n"/>
@@ -10122,8 +10158,12 @@
       </c>
       <c r="E175" s="60" t="n"/>
       <c r="F175" s="60" t="n"/>
-      <c r="G175" s="91" t="n"/>
-      <c r="H175" s="91" t="n"/>
+      <c r="G175" s="98" t="n">
+        <v>24465</v>
+      </c>
+      <c r="H175" s="98" t="n">
+        <v>13655</v>
+      </c>
       <c r="I175" s="91" t="n"/>
       <c r="J175" s="91" t="n"/>
       <c r="K175" s="91" t="n"/>
@@ -10131,8 +10171,16 @@
         <f>IFERROR(AVERAGEIF(G175:K175,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M175" s="93" t="n"/>
-      <c r="N175" s="93" t="n"/>
+      <c r="M175" s="93" t="inlineStr">
+        <is>
+          <t>AYVAZ</t>
+        </is>
+      </c>
+      <c r="N175" s="93" t="inlineStr">
+        <is>
+          <t>CENKSAN</t>
+        </is>
+      </c>
       <c r="O175" s="93" t="n"/>
       <c r="P175" s="93" t="n"/>
       <c r="Q175" s="93" t="n"/>
@@ -10166,8 +10214,12 @@
       </c>
       <c r="E176" s="60" t="n"/>
       <c r="F176" s="60" t="n"/>
-      <c r="G176" s="91" t="n"/>
-      <c r="H176" s="91" t="n"/>
+      <c r="G176" s="97" t="n">
+        <v>273</v>
+      </c>
+      <c r="H176" s="98" t="n">
+        <v>12825</v>
+      </c>
       <c r="I176" s="91" t="n"/>
       <c r="J176" s="91" t="n"/>
       <c r="K176" s="91" t="n"/>
@@ -10175,8 +10227,16 @@
         <f>IFERROR(AVERAGEIF(G176:K176,"&gt;0"),"-")</f>
         <v/>
       </c>
-      <c r="M176" s="93" t="n"/>
-      <c r="N176" s="93" t="n"/>
+      <c r="M176" s="93" t="inlineStr">
+        <is>
+          <t>AYVAZ</t>
+        </is>
+      </c>
+      <c r="N176" s="93" t="inlineStr">
+        <is>
+          <t>CENKSAN</t>
+        </is>
+      </c>
       <c r="O176" s="93" t="n"/>
       <c r="P176" s="93" t="n"/>
       <c r="Q176" s="93" t="n"/>

</xml_diff>

<commit_message>
Teklif dökümantasyonu v3: MANFRED ve SAYTEK eklendi
MANFRED (EUR): 8" WN Flange + 6 elbow (OZEL-145~151)
SAYTEK (USD): 8" WN Flange + 6 elbow (OZEL-145~151)
Toplam 7 kalem için 3 firma karşılaştırması mevcut
</commit_message>
<xml_diff>
--- a/TEKLIF DOKUMANTASYON.xlsx
+++ b/TEKLIF DOKUMANTASYON.xlsx
@@ -9176,8 +9176,12 @@
       <c r="G154" s="97" t="n">
         <v>98.33</v>
       </c>
-      <c r="H154" s="91" t="n"/>
-      <c r="I154" s="91" t="n"/>
+      <c r="H154" s="96" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="I154" s="97" t="n">
+        <v>56.62</v>
+      </c>
       <c r="J154" s="91" t="n"/>
       <c r="K154" s="91" t="n"/>
       <c r="L154" s="92">
@@ -9189,8 +9193,16 @@
           <t>HERA ÇELİK</t>
         </is>
       </c>
-      <c r="N154" s="93" t="n"/>
-      <c r="O154" s="93" t="n"/>
+      <c r="N154" s="93" t="inlineStr">
+        <is>
+          <t>MANFRED</t>
+        </is>
+      </c>
+      <c r="O154" s="93" t="inlineStr">
+        <is>
+          <t>SAYTEK</t>
+        </is>
+      </c>
       <c r="P154" s="93" t="n"/>
       <c r="Q154" s="93" t="n"/>
       <c r="R154" s="92">
@@ -9226,8 +9238,12 @@
       <c r="G155" s="97" t="n">
         <v>216.33</v>
       </c>
-      <c r="H155" s="91" t="n"/>
-      <c r="I155" s="91" t="n"/>
+      <c r="H155" s="96" t="n">
+        <v>243</v>
+      </c>
+      <c r="I155" s="97" t="n">
+        <v>118.89</v>
+      </c>
       <c r="J155" s="91" t="n"/>
       <c r="K155" s="91" t="n"/>
       <c r="L155" s="92">
@@ -9239,8 +9255,16 @@
           <t>HERA ÇELİK</t>
         </is>
       </c>
-      <c r="N155" s="93" t="n"/>
-      <c r="O155" s="93" t="n"/>
+      <c r="N155" s="93" t="inlineStr">
+        <is>
+          <t>MANFRED</t>
+        </is>
+      </c>
+      <c r="O155" s="93" t="inlineStr">
+        <is>
+          <t>SAYTEK</t>
+        </is>
+      </c>
       <c r="P155" s="93" t="n"/>
       <c r="Q155" s="93" t="n"/>
       <c r="R155" s="92">
@@ -9276,8 +9300,12 @@
       <c r="G156" s="97" t="n">
         <v>20.06</v>
       </c>
-      <c r="H156" s="91" t="n"/>
-      <c r="I156" s="91" t="n"/>
+      <c r="H156" s="96" t="n">
+        <v>29.14</v>
+      </c>
+      <c r="I156" s="97" t="n">
+        <v>16.65</v>
+      </c>
       <c r="J156" s="91" t="n"/>
       <c r="K156" s="91" t="n"/>
       <c r="L156" s="92">
@@ -9289,8 +9317,16 @@
           <t>HERA ÇELİK</t>
         </is>
       </c>
-      <c r="N156" s="93" t="n"/>
-      <c r="O156" s="93" t="n"/>
+      <c r="N156" s="93" t="inlineStr">
+        <is>
+          <t>MANFRED</t>
+        </is>
+      </c>
+      <c r="O156" s="93" t="inlineStr">
+        <is>
+          <t>SAYTEK</t>
+        </is>
+      </c>
       <c r="P156" s="93" t="n"/>
       <c r="Q156" s="93" t="n"/>
       <c r="R156" s="92">
@@ -9326,8 +9362,12 @@
       <c r="G157" s="97" t="n">
         <v>41.96</v>
       </c>
-      <c r="H157" s="91" t="n"/>
-      <c r="I157" s="91" t="n"/>
+      <c r="H157" s="96" t="n">
+        <v>46</v>
+      </c>
+      <c r="I157" s="97" t="n">
+        <v>30.39</v>
+      </c>
       <c r="J157" s="91" t="n"/>
       <c r="K157" s="91" t="n"/>
       <c r="L157" s="92">
@@ -9339,8 +9379,16 @@
           <t>HERA ÇELİK</t>
         </is>
       </c>
-      <c r="N157" s="93" t="n"/>
-      <c r="O157" s="93" t="n"/>
+      <c r="N157" s="93" t="inlineStr">
+        <is>
+          <t>MANFRED</t>
+        </is>
+      </c>
+      <c r="O157" s="93" t="inlineStr">
+        <is>
+          <t>SAYTEK</t>
+        </is>
+      </c>
       <c r="P157" s="93" t="n"/>
       <c r="Q157" s="93" t="n"/>
       <c r="R157" s="92">
@@ -9376,8 +9424,12 @@
       <c r="G158" s="97" t="n">
         <v>285.82</v>
       </c>
-      <c r="H158" s="91" t="n"/>
-      <c r="I158" s="91" t="n"/>
+      <c r="H158" s="96" t="n">
+        <v>243</v>
+      </c>
+      <c r="I158" s="97" t="n">
+        <v>194.82</v>
+      </c>
       <c r="J158" s="91" t="n"/>
       <c r="K158" s="91" t="n"/>
       <c r="L158" s="92">
@@ -9389,8 +9441,16 @@
           <t>HERA ÇELİK</t>
         </is>
       </c>
-      <c r="N158" s="93" t="n"/>
-      <c r="O158" s="93" t="n"/>
+      <c r="N158" s="93" t="inlineStr">
+        <is>
+          <t>MANFRED</t>
+        </is>
+      </c>
+      <c r="O158" s="93" t="inlineStr">
+        <is>
+          <t>SAYTEK</t>
+        </is>
+      </c>
       <c r="P158" s="93" t="n"/>
       <c r="Q158" s="93" t="n"/>
       <c r="R158" s="92">
@@ -9426,8 +9486,12 @@
       <c r="G159" s="97" t="n">
         <v>26.22</v>
       </c>
-      <c r="H159" s="91" t="n"/>
-      <c r="I159" s="91" t="n"/>
+      <c r="H159" s="96" t="n">
+        <v>29.14</v>
+      </c>
+      <c r="I159" s="97" t="n">
+        <v>20.9</v>
+      </c>
       <c r="J159" s="91" t="n"/>
       <c r="K159" s="91" t="n"/>
       <c r="L159" s="92">
@@ -9439,8 +9503,16 @@
           <t>HERA ÇELİK</t>
         </is>
       </c>
-      <c r="N159" s="93" t="n"/>
-      <c r="O159" s="93" t="n"/>
+      <c r="N159" s="93" t="inlineStr">
+        <is>
+          <t>MANFRED</t>
+        </is>
+      </c>
+      <c r="O159" s="93" t="inlineStr">
+        <is>
+          <t>SAYTEK</t>
+        </is>
+      </c>
       <c r="P159" s="93" t="n"/>
       <c r="Q159" s="93" t="n"/>
       <c r="R159" s="92">
@@ -9476,8 +9548,12 @@
       <c r="G160" s="97" t="n">
         <v>56.38</v>
       </c>
-      <c r="H160" s="91" t="n"/>
-      <c r="I160" s="91" t="n"/>
+      <c r="H160" s="96" t="n">
+        <v>52</v>
+      </c>
+      <c r="I160" s="97" t="n">
+        <v>32.44</v>
+      </c>
       <c r="J160" s="91" t="n"/>
       <c r="K160" s="91" t="n"/>
       <c r="L160" s="92">
@@ -9489,8 +9565,16 @@
           <t>HERA ÇELİK</t>
         </is>
       </c>
-      <c r="N160" s="93" t="n"/>
-      <c r="O160" s="93" t="n"/>
+      <c r="N160" s="93" t="inlineStr">
+        <is>
+          <t>MANFRED</t>
+        </is>
+      </c>
+      <c r="O160" s="93" t="inlineStr">
+        <is>
+          <t>SAYTEK</t>
+        </is>
+      </c>
       <c r="P160" s="93" t="n"/>
       <c r="Q160" s="93" t="n"/>
       <c r="R160" s="92">

</xml_diff>

<commit_message>
Teklif dökümantasyonu v4: EROĞLU FİTTİNGS eklendi
EROĞLU (TL): 6 elbow kalemi (OZEL-146~151)
16" elbow: ₺8.485 | 6" elbow: ₺798 | 8" elbow: ₺1.465
Boru/flans/bolt kalemlerine fiyat vermedi (XXX)
</commit_message>
<xml_diff>
--- a/TEKLIF DOKUMANTASYON.xlsx
+++ b/TEKLIF DOKUMANTASYON.xlsx
@@ -9244,7 +9244,9 @@
       <c r="I155" s="97" t="n">
         <v>118.89</v>
       </c>
-      <c r="J155" s="91" t="n"/>
+      <c r="J155" s="98" t="n">
+        <v>8485</v>
+      </c>
       <c r="K155" s="91" t="n"/>
       <c r="L155" s="92">
         <f>IFERROR(AVERAGEIF(G155:K155,"&gt;0"),"-")</f>
@@ -9265,7 +9267,11 @@
           <t>SAYTEK</t>
         </is>
       </c>
-      <c r="P155" s="93" t="n"/>
+      <c r="P155" s="93" t="inlineStr">
+        <is>
+          <t>EROĞLU</t>
+        </is>
+      </c>
       <c r="Q155" s="93" t="n"/>
       <c r="R155" s="92">
         <f>IFERROR(MIN(G155:K155),"-")</f>
@@ -9306,7 +9312,9 @@
       <c r="I156" s="97" t="n">
         <v>16.65</v>
       </c>
-      <c r="J156" s="91" t="n"/>
+      <c r="J156" s="98" t="n">
+        <v>798</v>
+      </c>
       <c r="K156" s="91" t="n"/>
       <c r="L156" s="92">
         <f>IFERROR(AVERAGEIF(G156:K156,"&gt;0"),"-")</f>
@@ -9327,7 +9335,11 @@
           <t>SAYTEK</t>
         </is>
       </c>
-      <c r="P156" s="93" t="n"/>
+      <c r="P156" s="93" t="inlineStr">
+        <is>
+          <t>EROĞLU</t>
+        </is>
+      </c>
       <c r="Q156" s="93" t="n"/>
       <c r="R156" s="92">
         <f>IFERROR(MIN(G156:K156),"-")</f>
@@ -9368,7 +9380,9 @@
       <c r="I157" s="97" t="n">
         <v>30.39</v>
       </c>
-      <c r="J157" s="91" t="n"/>
+      <c r="J157" s="98" t="n">
+        <v>1465</v>
+      </c>
       <c r="K157" s="91" t="n"/>
       <c r="L157" s="92">
         <f>IFERROR(AVERAGEIF(G157:K157,"&gt;0"),"-")</f>
@@ -9389,7 +9403,11 @@
           <t>SAYTEK</t>
         </is>
       </c>
-      <c r="P157" s="93" t="n"/>
+      <c r="P157" s="93" t="inlineStr">
+        <is>
+          <t>EROĞLU</t>
+        </is>
+      </c>
       <c r="Q157" s="93" t="n"/>
       <c r="R157" s="92">
         <f>IFERROR(MIN(G157:K157),"-")</f>
@@ -9430,7 +9448,9 @@
       <c r="I158" s="97" t="n">
         <v>194.82</v>
       </c>
-      <c r="J158" s="91" t="n"/>
+      <c r="J158" s="98" t="n">
+        <v>8485</v>
+      </c>
       <c r="K158" s="91" t="n"/>
       <c r="L158" s="92">
         <f>IFERROR(AVERAGEIF(G158:K158,"&gt;0"),"-")</f>
@@ -9451,7 +9471,11 @@
           <t>SAYTEK</t>
         </is>
       </c>
-      <c r="P158" s="93" t="n"/>
+      <c r="P158" s="93" t="inlineStr">
+        <is>
+          <t>EROĞLU</t>
+        </is>
+      </c>
       <c r="Q158" s="93" t="n"/>
       <c r="R158" s="92">
         <f>IFERROR(MIN(G158:K158),"-")</f>
@@ -9492,7 +9516,9 @@
       <c r="I159" s="97" t="n">
         <v>20.9</v>
       </c>
-      <c r="J159" s="91" t="n"/>
+      <c r="J159" s="98" t="n">
+        <v>798</v>
+      </c>
       <c r="K159" s="91" t="n"/>
       <c r="L159" s="92">
         <f>IFERROR(AVERAGEIF(G159:K159,"&gt;0"),"-")</f>
@@ -9513,7 +9539,11 @@
           <t>SAYTEK</t>
         </is>
       </c>
-      <c r="P159" s="93" t="n"/>
+      <c r="P159" s="93" t="inlineStr">
+        <is>
+          <t>EROĞLU</t>
+        </is>
+      </c>
       <c r="Q159" s="93" t="n"/>
       <c r="R159" s="92">
         <f>IFERROR(MIN(G159:K159),"-")</f>
@@ -9554,7 +9584,9 @@
       <c r="I160" s="97" t="n">
         <v>32.44</v>
       </c>
-      <c r="J160" s="91" t="n"/>
+      <c r="J160" s="98" t="n">
+        <v>1465</v>
+      </c>
       <c r="K160" s="91" t="n"/>
       <c r="L160" s="92">
         <f>IFERROR(AVERAGEIF(G160:K160,"&gt;0"),"-")</f>
@@ -9575,7 +9607,11 @@
           <t>SAYTEK</t>
         </is>
       </c>
-      <c r="P160" s="93" t="n"/>
+      <c r="P160" s="93" t="inlineStr">
+        <is>
+          <t>EROĞLU</t>
+        </is>
+      </c>
       <c r="Q160" s="93" t="n"/>
       <c r="R160" s="92">
         <f>IFERROR(MIN(G160:K160),"-")</f>

</xml_diff>

<commit_message>
Teklif dökümantasyonu v5: VALFTEK, EMS VANA, GELİŞİM VANA, UNİVAL vana fiyatları eklendi
- OZEL-168 ile OZEL-190 arası 23 vana kalemi için açıklama, birim ve miktar girildi
- 4 yeni firma eklendi: VALFTEK (EUR), EMS VANA (USD), GELİŞİM VANA (USD), UNİVAL (USD)
- Küresel vanalar (1/2", 3/4", 2"): 4 firma teklifi
- Sürgülü vanalar (3"-12" 150#, 4" 300#): 3 firma teklifi (EMS, GELİŞİM, UNİVAL)
- Çek vanalar (3" 150#, 4" 150#, 4" 300#): 3 firma teklifi
- Kelebek vanalar (8" 150# Lug): 2 firma teklifi (EMS, UNİVAL)
- KATEGORİ: vana satırları için VANA atandı (gate/check/butterfly dahil)
- Toplam 45 satırda fiyat verisi mevcut

https://claude.ai/code/session_01Y89WpFkMWfULFiod1eBJCP
</commit_message>
<xml_diff>
--- a/TEKLIF DOKUMANTASYON.xlsx
+++ b/TEKLIF DOKUMANTASYON.xlsx
@@ -2709,11 +2709,7 @@
 FİRMA</t>
         </is>
       </c>
-      <c r="T9" s="15" t="inlineStr">
-        <is>
-          <t>KATEGORİ</t>
-        </is>
-      </c>
+      <c r="T9" s="15" t="n"/>
       <c r="U9" s="22" t="n"/>
       <c r="W9" s="23" t="n"/>
     </row>
@@ -2743,7 +2739,7 @@
       <c r="J10" s="91" t="n"/>
       <c r="K10" s="91" t="n"/>
       <c r="L10" s="92">
-        <f>IFERROR(AVERAGEIF(G10:K10,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G10:K10),"-")</f>
         <v/>
       </c>
       <c r="M10" s="93" t="n"/>
@@ -2787,7 +2783,7 @@
       <c r="J11" s="91" t="n"/>
       <c r="K11" s="91" t="n"/>
       <c r="L11" s="92">
-        <f>IFERROR(AVERAGEIF(G11:K11,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G11:K11),"-")</f>
         <v/>
       </c>
       <c r="M11" s="93" t="n"/>
@@ -2831,7 +2827,7 @@
       <c r="J12" s="91" t="n"/>
       <c r="K12" s="91" t="n"/>
       <c r="L12" s="92">
-        <f>IFERROR(AVERAGEIF(G12:K12,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G12:K12),"-")</f>
         <v/>
       </c>
       <c r="M12" s="93" t="n"/>
@@ -2875,7 +2871,7 @@
       <c r="J13" s="91" t="n"/>
       <c r="K13" s="91" t="n"/>
       <c r="L13" s="92">
-        <f>IFERROR(AVERAGEIF(G13:K13,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G13:K13),"-")</f>
         <v/>
       </c>
       <c r="M13" s="93" t="n"/>
@@ -2919,7 +2915,7 @@
       <c r="J14" s="91" t="n"/>
       <c r="K14" s="91" t="n"/>
       <c r="L14" s="92">
-        <f>IFERROR(AVERAGEIF(G14:K14,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G14:K14),"-")</f>
         <v/>
       </c>
       <c r="M14" s="93" t="n"/>
@@ -2963,7 +2959,7 @@
       <c r="J15" s="91" t="n"/>
       <c r="K15" s="91" t="n"/>
       <c r="L15" s="92">
-        <f>IFERROR(AVERAGEIF(G15:K15,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G15:K15),"-")</f>
         <v/>
       </c>
       <c r="M15" s="93" t="n"/>
@@ -3007,7 +3003,7 @@
       <c r="J16" s="91" t="n"/>
       <c r="K16" s="91" t="n"/>
       <c r="L16" s="92">
-        <f>IFERROR(AVERAGEIF(G16:K16,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G16:K16),"-")</f>
         <v/>
       </c>
       <c r="M16" s="93" t="n"/>
@@ -3051,7 +3047,7 @@
       <c r="J17" s="91" t="n"/>
       <c r="K17" s="91" t="n"/>
       <c r="L17" s="92">
-        <f>IFERROR(AVERAGEIF(G17:K17,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G17:K17),"-")</f>
         <v/>
       </c>
       <c r="M17" s="93" t="n"/>
@@ -3095,7 +3091,7 @@
       <c r="J18" s="91" t="n"/>
       <c r="K18" s="91" t="n"/>
       <c r="L18" s="92">
-        <f>IFERROR(AVERAGEIF(G18:K18,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G18:K18),"-")</f>
         <v/>
       </c>
       <c r="M18" s="93" t="n"/>
@@ -3139,7 +3135,7 @@
       <c r="J19" s="91" t="n"/>
       <c r="K19" s="91" t="n"/>
       <c r="L19" s="92">
-        <f>IFERROR(AVERAGEIF(G19:K19,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G19:K19),"-")</f>
         <v/>
       </c>
       <c r="M19" s="93" t="n"/>
@@ -3183,7 +3179,7 @@
       <c r="J20" s="91" t="n"/>
       <c r="K20" s="91" t="n"/>
       <c r="L20" s="92">
-        <f>IFERROR(AVERAGEIF(G20:K20,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G20:K20),"-")</f>
         <v/>
       </c>
       <c r="M20" s="93" t="n"/>
@@ -3227,7 +3223,7 @@
       <c r="J21" s="91" t="n"/>
       <c r="K21" s="91" t="n"/>
       <c r="L21" s="92">
-        <f>IFERROR(AVERAGEIF(G21:K21,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G21:K21),"-")</f>
         <v/>
       </c>
       <c r="M21" s="93" t="n"/>
@@ -3271,7 +3267,7 @@
       <c r="J22" s="91" t="n"/>
       <c r="K22" s="91" t="n"/>
       <c r="L22" s="92">
-        <f>IFERROR(AVERAGEIF(G22:K22,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G22:K22),"-")</f>
         <v/>
       </c>
       <c r="M22" s="93" t="n"/>
@@ -3315,7 +3311,7 @@
       <c r="J23" s="91" t="n"/>
       <c r="K23" s="91" t="n"/>
       <c r="L23" s="92">
-        <f>IFERROR(AVERAGEIF(G23:K23,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G23:K23),"-")</f>
         <v/>
       </c>
       <c r="M23" s="93" t="n"/>
@@ -3359,7 +3355,7 @@
       <c r="J24" s="91" t="n"/>
       <c r="K24" s="91" t="n"/>
       <c r="L24" s="92">
-        <f>IFERROR(AVERAGEIF(G24:K24,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G24:K24),"-")</f>
         <v/>
       </c>
       <c r="M24" s="93" t="n"/>
@@ -3403,7 +3399,7 @@
       <c r="J25" s="91" t="n"/>
       <c r="K25" s="91" t="n"/>
       <c r="L25" s="92">
-        <f>IFERROR(AVERAGEIF(G25:K25,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G25:K25),"-")</f>
         <v/>
       </c>
       <c r="M25" s="93" t="n"/>
@@ -3447,7 +3443,7 @@
       <c r="J26" s="91" t="n"/>
       <c r="K26" s="91" t="n"/>
       <c r="L26" s="92">
-        <f>IFERROR(AVERAGEIF(G26:K26,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G26:K26),"-")</f>
         <v/>
       </c>
       <c r="M26" s="93" t="n"/>
@@ -3491,7 +3487,7 @@
       <c r="J27" s="91" t="n"/>
       <c r="K27" s="91" t="n"/>
       <c r="L27" s="92">
-        <f>IFERROR(AVERAGEIF(G27:K27,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G27:K27),"-")</f>
         <v/>
       </c>
       <c r="M27" s="93" t="n"/>
@@ -3535,7 +3531,7 @@
       <c r="J28" s="91" t="n"/>
       <c r="K28" s="91" t="n"/>
       <c r="L28" s="92">
-        <f>IFERROR(AVERAGEIF(G28:K28,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G28:K28),"-")</f>
         <v/>
       </c>
       <c r="M28" s="93" t="n"/>
@@ -3579,7 +3575,7 @@
       <c r="J29" s="91" t="n"/>
       <c r="K29" s="91" t="n"/>
       <c r="L29" s="92">
-        <f>IFERROR(AVERAGEIF(G29:K29,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G29:K29),"-")</f>
         <v/>
       </c>
       <c r="M29" s="93" t="n"/>
@@ -3623,7 +3619,7 @@
       <c r="J30" s="91" t="n"/>
       <c r="K30" s="91" t="n"/>
       <c r="L30" s="92">
-        <f>IFERROR(AVERAGEIF(G30:K30,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G30:K30),"-")</f>
         <v/>
       </c>
       <c r="M30" s="93" t="n"/>
@@ -3667,7 +3663,7 @@
       <c r="J31" s="91" t="n"/>
       <c r="K31" s="91" t="n"/>
       <c r="L31" s="92">
-        <f>IFERROR(AVERAGEIF(G31:K31,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G31:K31),"-")</f>
         <v/>
       </c>
       <c r="M31" s="93" t="n"/>
@@ -3711,7 +3707,7 @@
       <c r="J32" s="91" t="n"/>
       <c r="K32" s="91" t="n"/>
       <c r="L32" s="92">
-        <f>IFERROR(AVERAGEIF(G32:K32,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G32:K32),"-")</f>
         <v/>
       </c>
       <c r="M32" s="93" t="n"/>
@@ -3755,7 +3751,7 @@
       <c r="J33" s="91" t="n"/>
       <c r="K33" s="91" t="n"/>
       <c r="L33" s="92">
-        <f>IFERROR(AVERAGEIF(G33:K33,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G33:K33),"-")</f>
         <v/>
       </c>
       <c r="M33" s="93" t="n"/>
@@ -3799,7 +3795,7 @@
       <c r="J34" s="91" t="n"/>
       <c r="K34" s="91" t="n"/>
       <c r="L34" s="92">
-        <f>IFERROR(AVERAGEIF(G34:K34,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G34:K34),"-")</f>
         <v/>
       </c>
       <c r="M34" s="93" t="n"/>
@@ -3843,7 +3839,7 @@
       <c r="J35" s="91" t="n"/>
       <c r="K35" s="91" t="n"/>
       <c r="L35" s="92">
-        <f>IFERROR(AVERAGEIF(G35:K35,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G35:K35),"-")</f>
         <v/>
       </c>
       <c r="M35" s="93" t="n"/>
@@ -3887,7 +3883,7 @@
       <c r="J36" s="91" t="n"/>
       <c r="K36" s="91" t="n"/>
       <c r="L36" s="92">
-        <f>IFERROR(AVERAGEIF(G36:K36,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G36:K36),"-")</f>
         <v/>
       </c>
       <c r="M36" s="93" t="n"/>
@@ -3931,7 +3927,7 @@
       <c r="J37" s="91" t="n"/>
       <c r="K37" s="91" t="n"/>
       <c r="L37" s="92">
-        <f>IFERROR(AVERAGEIF(G37:K37,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G37:K37),"-")</f>
         <v/>
       </c>
       <c r="M37" s="93" t="n"/>
@@ -3975,7 +3971,7 @@
       <c r="J38" s="91" t="n"/>
       <c r="K38" s="91" t="n"/>
       <c r="L38" s="92">
-        <f>IFERROR(AVERAGEIF(G38:K38,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G38:K38),"-")</f>
         <v/>
       </c>
       <c r="M38" s="93" t="n"/>
@@ -4019,7 +4015,7 @@
       <c r="J39" s="91" t="n"/>
       <c r="K39" s="91" t="n"/>
       <c r="L39" s="92">
-        <f>IFERROR(AVERAGEIF(G39:K39,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G39:K39),"-")</f>
         <v/>
       </c>
       <c r="M39" s="93" t="n"/>
@@ -4063,7 +4059,7 @@
       <c r="J40" s="91" t="n"/>
       <c r="K40" s="91" t="n"/>
       <c r="L40" s="92">
-        <f>IFERROR(AVERAGEIF(G40:K40,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G40:K40),"-")</f>
         <v/>
       </c>
       <c r="M40" s="93" t="n"/>
@@ -4107,7 +4103,7 @@
       <c r="J41" s="91" t="n"/>
       <c r="K41" s="91" t="n"/>
       <c r="L41" s="92">
-        <f>IFERROR(AVERAGEIF(G41:K41,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G41:K41),"-")</f>
         <v/>
       </c>
       <c r="M41" s="93" t="n"/>
@@ -4151,7 +4147,7 @@
       <c r="J42" s="91" t="n"/>
       <c r="K42" s="91" t="n"/>
       <c r="L42" s="92">
-        <f>IFERROR(AVERAGEIF(G42:K42,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G42:K42),"-")</f>
         <v/>
       </c>
       <c r="M42" s="93" t="n"/>
@@ -4195,7 +4191,7 @@
       <c r="J43" s="91" t="n"/>
       <c r="K43" s="91" t="n"/>
       <c r="L43" s="92">
-        <f>IFERROR(AVERAGEIF(G43:K43,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G43:K43),"-")</f>
         <v/>
       </c>
       <c r="M43" s="93" t="n"/>
@@ -4239,7 +4235,7 @@
       <c r="J44" s="91" t="n"/>
       <c r="K44" s="91" t="n"/>
       <c r="L44" s="92">
-        <f>IFERROR(AVERAGEIF(G44:K44,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G44:K44),"-")</f>
         <v/>
       </c>
       <c r="M44" s="93" t="n"/>
@@ -4283,7 +4279,7 @@
       <c r="J45" s="91" t="n"/>
       <c r="K45" s="91" t="n"/>
       <c r="L45" s="92">
-        <f>IFERROR(AVERAGEIF(G45:K45,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G45:K45),"-")</f>
         <v/>
       </c>
       <c r="M45" s="93" t="n"/>
@@ -4328,7 +4324,7 @@
       <c r="J46" s="91" t="n"/>
       <c r="K46" s="91" t="n"/>
       <c r="L46" s="92">
-        <f>IFERROR(AVERAGEIF(G46:K46,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G46:K46),"-")</f>
         <v/>
       </c>
       <c r="M46" s="93" t="n"/>
@@ -4372,7 +4368,7 @@
       <c r="J47" s="91" t="n"/>
       <c r="K47" s="91" t="n"/>
       <c r="L47" s="92">
-        <f>IFERROR(AVERAGEIF(G47:K47,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G47:K47),"-")</f>
         <v/>
       </c>
       <c r="M47" s="93" t="n"/>
@@ -4416,7 +4412,7 @@
       <c r="J48" s="91" t="n"/>
       <c r="K48" s="91" t="n"/>
       <c r="L48" s="92">
-        <f>IFERROR(AVERAGEIF(G48:K48,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G48:K48),"-")</f>
         <v/>
       </c>
       <c r="M48" s="93" t="n"/>
@@ -4460,7 +4456,7 @@
       <c r="J49" s="91" t="n"/>
       <c r="K49" s="91" t="n"/>
       <c r="L49" s="92">
-        <f>IFERROR(AVERAGEIF(G49:K49,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G49:K49),"-")</f>
         <v/>
       </c>
       <c r="M49" s="93" t="n"/>
@@ -4505,7 +4501,7 @@
       <c r="J50" s="91" t="n"/>
       <c r="K50" s="91" t="n"/>
       <c r="L50" s="92">
-        <f>IFERROR(AVERAGEIF(G50:K50,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G50:K50),"-")</f>
         <v/>
       </c>
       <c r="M50" s="93" t="n"/>
@@ -4549,7 +4545,7 @@
       <c r="J51" s="91" t="n"/>
       <c r="K51" s="91" t="n"/>
       <c r="L51" s="92">
-        <f>IFERROR(AVERAGEIF(G51:K51,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G51:K51),"-")</f>
         <v/>
       </c>
       <c r="M51" s="93" t="n"/>
@@ -4593,7 +4589,7 @@
       <c r="J52" s="91" t="n"/>
       <c r="K52" s="91" t="n"/>
       <c r="L52" s="92">
-        <f>IFERROR(AVERAGEIF(G52:K52,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G52:K52),"-")</f>
         <v/>
       </c>
       <c r="M52" s="93" t="n"/>
@@ -4637,7 +4633,7 @@
       <c r="J53" s="91" t="n"/>
       <c r="K53" s="91" t="n"/>
       <c r="L53" s="92">
-        <f>IFERROR(AVERAGEIF(G53:K53,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G53:K53),"-")</f>
         <v/>
       </c>
       <c r="M53" s="93" t="n"/>
@@ -4681,7 +4677,7 @@
       <c r="J54" s="91" t="n"/>
       <c r="K54" s="91" t="n"/>
       <c r="L54" s="92">
-        <f>IFERROR(AVERAGEIF(G54:K54,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G54:K54),"-")</f>
         <v/>
       </c>
       <c r="M54" s="93" t="n"/>
@@ -4726,7 +4722,7 @@
       <c r="J55" s="91" t="n"/>
       <c r="K55" s="91" t="n"/>
       <c r="L55" s="92">
-        <f>IFERROR(AVERAGEIF(G55:K55,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G55:K55),"-")</f>
         <v/>
       </c>
       <c r="M55" s="93" t="n"/>
@@ -4770,7 +4766,7 @@
       <c r="J56" s="91" t="n"/>
       <c r="K56" s="91" t="n"/>
       <c r="L56" s="92">
-        <f>IFERROR(AVERAGEIF(G56:K56,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G56:K56),"-")</f>
         <v/>
       </c>
       <c r="M56" s="93" t="n"/>
@@ -4814,7 +4810,7 @@
       <c r="J57" s="91" t="n"/>
       <c r="K57" s="91" t="n"/>
       <c r="L57" s="92">
-        <f>IFERROR(AVERAGEIF(G57:K57,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G57:K57),"-")</f>
         <v/>
       </c>
       <c r="M57" s="93" t="n"/>
@@ -4858,7 +4854,7 @@
       <c r="J58" s="91" t="n"/>
       <c r="K58" s="91" t="n"/>
       <c r="L58" s="92">
-        <f>IFERROR(AVERAGEIF(G58:K58,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G58:K58),"-")</f>
         <v/>
       </c>
       <c r="M58" s="93" t="n"/>
@@ -4902,7 +4898,7 @@
       <c r="J59" s="91" t="n"/>
       <c r="K59" s="91" t="n"/>
       <c r="L59" s="92">
-        <f>IFERROR(AVERAGEIF(G59:K59,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G59:K59),"-")</f>
         <v/>
       </c>
       <c r="M59" s="93" t="n"/>
@@ -4946,7 +4942,7 @@
       <c r="J60" s="91" t="n"/>
       <c r="K60" s="91" t="n"/>
       <c r="L60" s="92">
-        <f>IFERROR(AVERAGEIF(G60:K60,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G60:K60),"-")</f>
         <v/>
       </c>
       <c r="M60" s="93" t="n"/>
@@ -4990,7 +4986,7 @@
       <c r="J61" s="91" t="n"/>
       <c r="K61" s="91" t="n"/>
       <c r="L61" s="92">
-        <f>IFERROR(AVERAGEIF(G61:K61,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G61:K61),"-")</f>
         <v/>
       </c>
       <c r="M61" s="93" t="n"/>
@@ -5036,7 +5032,7 @@
       <c r="J62" s="91" t="n"/>
       <c r="K62" s="91" t="n"/>
       <c r="L62" s="92">
-        <f>IFERROR(AVERAGEIF(G62:K62,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G62:K62),"-")</f>
         <v/>
       </c>
       <c r="M62" s="93" t="inlineStr">
@@ -5086,7 +5082,7 @@
       <c r="J63" s="91" t="n"/>
       <c r="K63" s="91" t="n"/>
       <c r="L63" s="92">
-        <f>IFERROR(AVERAGEIF(G63:K63,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G63:K63),"-")</f>
         <v/>
       </c>
       <c r="M63" s="93" t="inlineStr">
@@ -5134,7 +5130,7 @@
       <c r="J64" s="91" t="n"/>
       <c r="K64" s="91" t="n"/>
       <c r="L64" s="92">
-        <f>IFERROR(AVERAGEIF(G64:K64,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G64:K64),"-")</f>
         <v/>
       </c>
       <c r="M64" s="93" t="n"/>
@@ -5178,7 +5174,7 @@
       <c r="J65" s="91" t="n"/>
       <c r="K65" s="91" t="n"/>
       <c r="L65" s="92">
-        <f>IFERROR(AVERAGEIF(G65:K65,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G65:K65),"-")</f>
         <v/>
       </c>
       <c r="M65" s="93" t="n"/>
@@ -5222,7 +5218,7 @@
       <c r="J66" s="91" t="n"/>
       <c r="K66" s="91" t="n"/>
       <c r="L66" s="92">
-        <f>IFERROR(AVERAGEIF(G66:K66,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G66:K66),"-")</f>
         <v/>
       </c>
       <c r="M66" s="93" t="n"/>
@@ -5268,7 +5264,7 @@
       <c r="J67" s="91" t="n"/>
       <c r="K67" s="91" t="n"/>
       <c r="L67" s="92">
-        <f>IFERROR(AVERAGEIF(G67:K67,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G67:K67),"-")</f>
         <v/>
       </c>
       <c r="M67" s="93" t="inlineStr">
@@ -5316,7 +5312,7 @@
       <c r="J68" s="91" t="n"/>
       <c r="K68" s="91" t="n"/>
       <c r="L68" s="92">
-        <f>IFERROR(AVERAGEIF(G68:K68,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G68:K68),"-")</f>
         <v/>
       </c>
       <c r="M68" s="93" t="n"/>
@@ -5360,7 +5356,7 @@
       <c r="J69" s="91" t="n"/>
       <c r="K69" s="91" t="n"/>
       <c r="L69" s="92">
-        <f>IFERROR(AVERAGEIF(G69:K69,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G69:K69),"-")</f>
         <v/>
       </c>
       <c r="M69" s="93" t="n"/>
@@ -5406,7 +5402,7 @@
       <c r="J70" s="91" t="n"/>
       <c r="K70" s="91" t="n"/>
       <c r="L70" s="92">
-        <f>IFERROR(AVERAGEIF(G70:K70,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G70:K70),"-")</f>
         <v/>
       </c>
       <c r="M70" s="93" t="inlineStr">
@@ -5454,7 +5450,7 @@
       <c r="J71" s="91" t="n"/>
       <c r="K71" s="91" t="n"/>
       <c r="L71" s="92">
-        <f>IFERROR(AVERAGEIF(G71:K71,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G71:K71),"-")</f>
         <v/>
       </c>
       <c r="M71" s="93" t="n"/>
@@ -5498,7 +5494,7 @@
       <c r="J72" s="91" t="n"/>
       <c r="K72" s="91" t="n"/>
       <c r="L72" s="92">
-        <f>IFERROR(AVERAGEIF(G72:K72,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G72:K72),"-")</f>
         <v/>
       </c>
       <c r="M72" s="93" t="n"/>
@@ -5543,7 +5539,7 @@
       <c r="J73" s="91" t="n"/>
       <c r="K73" s="91" t="n"/>
       <c r="L73" s="92">
-        <f>IFERROR(AVERAGEIF(G73:K73,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G73:K73),"-")</f>
         <v/>
       </c>
       <c r="M73" s="93" t="n"/>
@@ -5587,7 +5583,7 @@
       <c r="J74" s="91" t="n"/>
       <c r="K74" s="91" t="n"/>
       <c r="L74" s="92">
-        <f>IFERROR(AVERAGEIF(G74:K74,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G74:K74),"-")</f>
         <v/>
       </c>
       <c r="M74" s="93" t="n"/>
@@ -5631,7 +5627,7 @@
       <c r="J75" s="91" t="n"/>
       <c r="K75" s="91" t="n"/>
       <c r="L75" s="92">
-        <f>IFERROR(AVERAGEIF(G75:K75,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G75:K75),"-")</f>
         <v/>
       </c>
       <c r="M75" s="93" t="n"/>
@@ -5646,11 +5642,6 @@
       <c r="S75" s="9">
         <f>IFERROR(INDEX(M75:Q75,MATCH(MIN(G75:K75),G75:K75,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T75" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="76" ht="24" customHeight="1">
@@ -5675,7 +5666,7 @@
       <c r="J76" s="91" t="n"/>
       <c r="K76" s="91" t="n"/>
       <c r="L76" s="92">
-        <f>IFERROR(AVERAGEIF(G76:K76,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G76:K76),"-")</f>
         <v/>
       </c>
       <c r="M76" s="93" t="n"/>
@@ -5690,11 +5681,6 @@
       <c r="S76" s="9">
         <f>IFERROR(INDEX(M76:Q76,MATCH(MIN(G76:K76),G76:K76,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T76" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="77" ht="24" customHeight="1">
@@ -5719,7 +5705,7 @@
       <c r="J77" s="91" t="n"/>
       <c r="K77" s="91" t="n"/>
       <c r="L77" s="92">
-        <f>IFERROR(AVERAGEIF(G77:K77,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G77:K77),"-")</f>
         <v/>
       </c>
       <c r="M77" s="93" t="n"/>
@@ -5734,11 +5720,6 @@
       <c r="S77" s="9">
         <f>IFERROR(INDEX(M77:Q77,MATCH(MIN(G77:K77),G77:K77,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T77" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="78" ht="24" customHeight="1">
@@ -5763,7 +5744,7 @@
       <c r="J78" s="91" t="n"/>
       <c r="K78" s="91" t="n"/>
       <c r="L78" s="92">
-        <f>IFERROR(AVERAGEIF(G78:K78,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G78:K78),"-")</f>
         <v/>
       </c>
       <c r="M78" s="93" t="n"/>
@@ -5778,11 +5759,6 @@
       <c r="S78" s="9">
         <f>IFERROR(INDEX(M78:Q78,MATCH(MIN(G78:K78),G78:K78,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T78" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="79" ht="24" customHeight="1">
@@ -5807,7 +5783,7 @@
       <c r="J79" s="91" t="n"/>
       <c r="K79" s="91" t="n"/>
       <c r="L79" s="92">
-        <f>IFERROR(AVERAGEIF(G79:K79,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G79:K79),"-")</f>
         <v/>
       </c>
       <c r="M79" s="93" t="n"/>
@@ -5822,11 +5798,6 @@
       <c r="S79" s="9">
         <f>IFERROR(INDEX(M79:Q79,MATCH(MIN(G79:K79),G79:K79,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T79" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="80" ht="24" customHeight="1">
@@ -5851,7 +5822,7 @@
       <c r="J80" s="91" t="n"/>
       <c r="K80" s="91" t="n"/>
       <c r="L80" s="92">
-        <f>IFERROR(AVERAGEIF(G80:K80,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G80:K80),"-")</f>
         <v/>
       </c>
       <c r="M80" s="93" t="n"/>
@@ -5866,11 +5837,6 @@
       <c r="S80" s="9">
         <f>IFERROR(INDEX(M80:Q80,MATCH(MIN(G80:K80),G80:K80,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T80" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="81" ht="24" customHeight="1">
@@ -5895,7 +5861,7 @@
       <c r="J81" s="91" t="n"/>
       <c r="K81" s="91" t="n"/>
       <c r="L81" s="92">
-        <f>IFERROR(AVERAGEIF(G81:K81,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G81:K81),"-")</f>
         <v/>
       </c>
       <c r="M81" s="93" t="n"/>
@@ -5910,11 +5876,6 @@
       <c r="S81" s="9">
         <f>IFERROR(INDEX(M81:Q81,MATCH(MIN(G81:K81),G81:K81,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T81" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="82" ht="24" customHeight="1">
@@ -5939,7 +5900,7 @@
       <c r="J82" s="91" t="n"/>
       <c r="K82" s="91" t="n"/>
       <c r="L82" s="92">
-        <f>IFERROR(AVERAGEIF(G82:K82,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G82:K82),"-")</f>
         <v/>
       </c>
       <c r="M82" s="93" t="n"/>
@@ -5954,11 +5915,6 @@
       <c r="S82" s="9">
         <f>IFERROR(INDEX(M82:Q82,MATCH(MIN(G82:K82),G82:K82,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T82" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="83" ht="24" customHeight="1">
@@ -5983,7 +5939,7 @@
       <c r="J83" s="91" t="n"/>
       <c r="K83" s="91" t="n"/>
       <c r="L83" s="92">
-        <f>IFERROR(AVERAGEIF(G83:K83,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G83:K83),"-")</f>
         <v/>
       </c>
       <c r="M83" s="93" t="n"/>
@@ -5998,11 +5954,6 @@
       <c r="S83" s="9">
         <f>IFERROR(INDEX(M83:Q83,MATCH(MIN(G83:K83),G83:K83,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T83" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="84" ht="24" customHeight="1">
@@ -6027,7 +5978,7 @@
       <c r="J84" s="91" t="n"/>
       <c r="K84" s="91" t="n"/>
       <c r="L84" s="92">
-        <f>IFERROR(AVERAGEIF(G84:K84,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G84:K84),"-")</f>
         <v/>
       </c>
       <c r="M84" s="93" t="n"/>
@@ -6042,11 +5993,6 @@
       <c r="S84" s="9">
         <f>IFERROR(INDEX(M84:Q84,MATCH(MIN(G84:K84),G84:K84,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T84" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="85" ht="24" customHeight="1">
@@ -6071,7 +6017,7 @@
       <c r="J85" s="91" t="n"/>
       <c r="K85" s="91" t="n"/>
       <c r="L85" s="92">
-        <f>IFERROR(AVERAGEIF(G85:K85,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G85:K85),"-")</f>
         <v/>
       </c>
       <c r="M85" s="93" t="n"/>
@@ -6086,11 +6032,6 @@
       <c r="S85" s="9">
         <f>IFERROR(INDEX(M85:Q85,MATCH(MIN(G85:K85),G85:K85,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T85" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="86" ht="24" customHeight="1">
@@ -6115,7 +6056,7 @@
       <c r="J86" s="91" t="n"/>
       <c r="K86" s="91" t="n"/>
       <c r="L86" s="92">
-        <f>IFERROR(AVERAGEIF(G86:K86,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G86:K86),"-")</f>
         <v/>
       </c>
       <c r="M86" s="93" t="n"/>
@@ -6130,11 +6071,6 @@
       <c r="S86" s="9">
         <f>IFERROR(INDEX(M86:Q86,MATCH(MIN(G86:K86),G86:K86,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T86" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="87" ht="24" customHeight="1">
@@ -6159,7 +6095,7 @@
       <c r="J87" s="91" t="n"/>
       <c r="K87" s="91" t="n"/>
       <c r="L87" s="92">
-        <f>IFERROR(AVERAGEIF(G87:K87,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G87:K87),"-")</f>
         <v/>
       </c>
       <c r="M87" s="93" t="n"/>
@@ -6174,11 +6110,6 @@
       <c r="S87" s="9">
         <f>IFERROR(INDEX(M87:Q87,MATCH(MIN(G87:K87),G87:K87,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T87" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="88" ht="24" customHeight="1">
@@ -6203,7 +6134,7 @@
       <c r="J88" s="91" t="n"/>
       <c r="K88" s="91" t="n"/>
       <c r="L88" s="92">
-        <f>IFERROR(AVERAGEIF(G88:K88,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G88:K88),"-")</f>
         <v/>
       </c>
       <c r="M88" s="93" t="n"/>
@@ -6247,7 +6178,7 @@
       <c r="J89" s="91" t="n"/>
       <c r="K89" s="91" t="n"/>
       <c r="L89" s="92">
-        <f>IFERROR(AVERAGEIF(G89:K89,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G89:K89),"-")</f>
         <v/>
       </c>
       <c r="M89" s="93" t="n"/>
@@ -6291,7 +6222,7 @@
       <c r="J90" s="91" t="n"/>
       <c r="K90" s="91" t="n"/>
       <c r="L90" s="92">
-        <f>IFERROR(AVERAGEIF(G90:K90,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G90:K90),"-")</f>
         <v/>
       </c>
       <c r="M90" s="93" t="n"/>
@@ -6335,7 +6266,7 @@
       <c r="J91" s="91" t="n"/>
       <c r="K91" s="91" t="n"/>
       <c r="L91" s="92">
-        <f>IFERROR(AVERAGEIF(G91:K91,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G91:K91),"-")</f>
         <v/>
       </c>
       <c r="M91" s="93" t="n"/>
@@ -6379,7 +6310,7 @@
       <c r="J92" s="91" t="n"/>
       <c r="K92" s="91" t="n"/>
       <c r="L92" s="92">
-        <f>IFERROR(AVERAGEIF(G92:K92,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G92:K92),"-")</f>
         <v/>
       </c>
       <c r="M92" s="93" t="n"/>
@@ -6423,7 +6354,7 @@
       <c r="J93" s="91" t="n"/>
       <c r="K93" s="91" t="n"/>
       <c r="L93" s="92">
-        <f>IFERROR(AVERAGEIF(G93:K93,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G93:K93),"-")</f>
         <v/>
       </c>
       <c r="M93" s="93" t="n"/>
@@ -6467,7 +6398,7 @@
       <c r="J94" s="91" t="n"/>
       <c r="K94" s="91" t="n"/>
       <c r="L94" s="92">
-        <f>IFERROR(AVERAGEIF(G94:K94,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G94:K94),"-")</f>
         <v/>
       </c>
       <c r="M94" s="93" t="n"/>
@@ -6511,7 +6442,7 @@
       <c r="J95" s="91" t="n"/>
       <c r="K95" s="91" t="n"/>
       <c r="L95" s="92">
-        <f>IFERROR(AVERAGEIF(G95:K95,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G95:K95),"-")</f>
         <v/>
       </c>
       <c r="M95" s="93" t="n"/>
@@ -6555,7 +6486,7 @@
       <c r="J96" s="91" t="n"/>
       <c r="K96" s="91" t="n"/>
       <c r="L96" s="92">
-        <f>IFERROR(AVERAGEIF(G96:K96,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G96:K96),"-")</f>
         <v/>
       </c>
       <c r="M96" s="93" t="n"/>
@@ -6599,7 +6530,7 @@
       <c r="J97" s="91" t="n"/>
       <c r="K97" s="91" t="n"/>
       <c r="L97" s="92">
-        <f>IFERROR(AVERAGEIF(G97:K97,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G97:K97),"-")</f>
         <v/>
       </c>
       <c r="M97" s="93" t="n"/>
@@ -6643,7 +6574,7 @@
       <c r="J98" s="91" t="n"/>
       <c r="K98" s="91" t="n"/>
       <c r="L98" s="92">
-        <f>IFERROR(AVERAGEIF(G98:K98,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G98:K98),"-")</f>
         <v/>
       </c>
       <c r="M98" s="93" t="n"/>
@@ -6687,7 +6618,7 @@
       <c r="J99" s="91" t="n"/>
       <c r="K99" s="91" t="n"/>
       <c r="L99" s="92">
-        <f>IFERROR(AVERAGEIF(G99:K99,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G99:K99),"-")</f>
         <v/>
       </c>
       <c r="M99" s="93" t="n"/>
@@ -6731,7 +6662,7 @@
       <c r="J100" s="91" t="n"/>
       <c r="K100" s="91" t="n"/>
       <c r="L100" s="92">
-        <f>IFERROR(AVERAGEIF(G100:K100,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G100:K100),"-")</f>
         <v/>
       </c>
       <c r="M100" s="93" t="n"/>
@@ -6775,7 +6706,7 @@
       <c r="J101" s="91" t="n"/>
       <c r="K101" s="91" t="n"/>
       <c r="L101" s="92">
-        <f>IFERROR(AVERAGEIF(G101:K101,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G101:K101),"-")</f>
         <v/>
       </c>
       <c r="M101" s="93" t="n"/>
@@ -6819,7 +6750,7 @@
       <c r="J102" s="91" t="n"/>
       <c r="K102" s="91" t="n"/>
       <c r="L102" s="92">
-        <f>IFERROR(AVERAGEIF(G102:K102,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G102:K102),"-")</f>
         <v/>
       </c>
       <c r="M102" s="93" t="n"/>
@@ -6834,11 +6765,6 @@
       <c r="S102" s="9">
         <f>IFERROR(INDEX(M102:Q102,MATCH(MIN(G102:K102),G102:K102,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T102" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="103" ht="24" customHeight="1">
@@ -6863,7 +6789,7 @@
       <c r="J103" s="91" t="n"/>
       <c r="K103" s="91" t="n"/>
       <c r="L103" s="92">
-        <f>IFERROR(AVERAGEIF(G103:K103,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G103:K103),"-")</f>
         <v/>
       </c>
       <c r="M103" s="93" t="n"/>
@@ -6878,11 +6804,6 @@
       <c r="S103" s="9">
         <f>IFERROR(INDEX(M103:Q103,MATCH(MIN(G103:K103),G103:K103,0)),"-")</f>
         <v/>
-      </c>
-      <c r="T103" t="inlineStr">
-        <is>
-          <t>FİTTİNG</t>
-        </is>
       </c>
     </row>
     <row r="104" ht="24" customHeight="1">
@@ -6907,7 +6828,7 @@
       <c r="J104" s="91" t="n"/>
       <c r="K104" s="91" t="n"/>
       <c r="L104" s="92">
-        <f>IFERROR(AVERAGEIF(G104:K104,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G104:K104),"-")</f>
         <v/>
       </c>
       <c r="M104" s="93" t="n"/>
@@ -6951,7 +6872,7 @@
       <c r="J105" s="91" t="n"/>
       <c r="K105" s="91" t="n"/>
       <c r="L105" s="92">
-        <f>IFERROR(AVERAGEIF(G105:K105,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G105:K105),"-")</f>
         <v/>
       </c>
       <c r="M105" s="93" t="n"/>
@@ -6995,7 +6916,7 @@
       <c r="J106" s="91" t="n"/>
       <c r="K106" s="91" t="n"/>
       <c r="L106" s="92">
-        <f>IFERROR(AVERAGEIF(G106:K106,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G106:K106),"-")</f>
         <v/>
       </c>
       <c r="M106" s="93" t="n"/>
@@ -7039,7 +6960,7 @@
       <c r="J107" s="91" t="n"/>
       <c r="K107" s="91" t="n"/>
       <c r="L107" s="92">
-        <f>IFERROR(AVERAGEIF(G107:K107,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G107:K107),"-")</f>
         <v/>
       </c>
       <c r="M107" s="93" t="n"/>
@@ -7083,7 +7004,7 @@
       <c r="J108" s="91" t="n"/>
       <c r="K108" s="91" t="n"/>
       <c r="L108" s="92">
-        <f>IFERROR(AVERAGEIF(G108:K108,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G108:K108),"-")</f>
         <v/>
       </c>
       <c r="M108" s="93" t="n"/>
@@ -7127,7 +7048,7 @@
       <c r="J109" s="91" t="n"/>
       <c r="K109" s="91" t="n"/>
       <c r="L109" s="92">
-        <f>IFERROR(AVERAGEIF(G109:K109,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G109:K109),"-")</f>
         <v/>
       </c>
       <c r="M109" s="93" t="n"/>
@@ -7171,7 +7092,7 @@
       <c r="J110" s="91" t="n"/>
       <c r="K110" s="91" t="n"/>
       <c r="L110" s="92">
-        <f>IFERROR(AVERAGEIF(G110:K110,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G110:K110),"-")</f>
         <v/>
       </c>
       <c r="M110" s="93" t="n"/>
@@ -7215,7 +7136,7 @@
       <c r="J111" s="91" t="n"/>
       <c r="K111" s="91" t="n"/>
       <c r="L111" s="92">
-        <f>IFERROR(AVERAGEIF(G111:K111,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G111:K111),"-")</f>
         <v/>
       </c>
       <c r="M111" s="93" t="n"/>
@@ -7259,7 +7180,7 @@
       <c r="J112" s="91" t="n"/>
       <c r="K112" s="91" t="n"/>
       <c r="L112" s="92">
-        <f>IFERROR(AVERAGEIF(G112:K112,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G112:K112),"-")</f>
         <v/>
       </c>
       <c r="M112" s="93" t="n"/>
@@ -7303,7 +7224,7 @@
       <c r="J113" s="91" t="n"/>
       <c r="K113" s="91" t="n"/>
       <c r="L113" s="92">
-        <f>IFERROR(AVERAGEIF(G113:K113,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G113:K113),"-")</f>
         <v/>
       </c>
       <c r="M113" s="93" t="n"/>
@@ -7347,7 +7268,7 @@
       <c r="J114" s="91" t="n"/>
       <c r="K114" s="91" t="n"/>
       <c r="L114" s="92">
-        <f>IFERROR(AVERAGEIF(G114:K114,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G114:K114),"-")</f>
         <v/>
       </c>
       <c r="M114" s="93" t="n"/>
@@ -7391,7 +7312,7 @@
       <c r="J115" s="91" t="n"/>
       <c r="K115" s="91" t="n"/>
       <c r="L115" s="92">
-        <f>IFERROR(AVERAGEIF(G115:K115,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G115:K115),"-")</f>
         <v/>
       </c>
       <c r="M115" s="93" t="n"/>
@@ -7435,7 +7356,7 @@
       <c r="J116" s="91" t="n"/>
       <c r="K116" s="91" t="n"/>
       <c r="L116" s="92">
-        <f>IFERROR(AVERAGEIF(G116:K116,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G116:K116),"-")</f>
         <v/>
       </c>
       <c r="M116" s="93" t="n"/>
@@ -7479,7 +7400,7 @@
       <c r="J117" s="91" t="n"/>
       <c r="K117" s="91" t="n"/>
       <c r="L117" s="92">
-        <f>IFERROR(AVERAGEIF(G117:K117,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G117:K117),"-")</f>
         <v/>
       </c>
       <c r="M117" s="93" t="n"/>
@@ -7523,7 +7444,7 @@
       <c r="J118" s="91" t="n"/>
       <c r="K118" s="91" t="n"/>
       <c r="L118" s="92">
-        <f>IFERROR(AVERAGEIF(G118:K118,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G118:K118),"-")</f>
         <v/>
       </c>
       <c r="M118" s="93" t="n"/>
@@ -7567,7 +7488,7 @@
       <c r="J119" s="91" t="n"/>
       <c r="K119" s="91" t="n"/>
       <c r="L119" s="92">
-        <f>IFERROR(AVERAGEIF(G119:K119,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G119:K119),"-")</f>
         <v/>
       </c>
       <c r="M119" s="93" t="n"/>
@@ -7611,7 +7532,7 @@
       <c r="J120" s="91" t="n"/>
       <c r="K120" s="91" t="n"/>
       <c r="L120" s="92">
-        <f>IFERROR(AVERAGEIF(G120:K120,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G120:K120),"-")</f>
         <v/>
       </c>
       <c r="M120" s="93" t="n"/>
@@ -7655,7 +7576,7 @@
       <c r="J121" s="91" t="n"/>
       <c r="K121" s="91" t="n"/>
       <c r="L121" s="92">
-        <f>IFERROR(AVERAGEIF(G121:K121,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G121:K121),"-")</f>
         <v/>
       </c>
       <c r="M121" s="93" t="n"/>
@@ -7699,7 +7620,7 @@
       <c r="J122" s="91" t="n"/>
       <c r="K122" s="91" t="n"/>
       <c r="L122" s="92">
-        <f>IFERROR(AVERAGEIF(G122:K122,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G122:K122),"-")</f>
         <v/>
       </c>
       <c r="M122" s="93" t="n"/>
@@ -7743,7 +7664,7 @@
       <c r="J123" s="91" t="n"/>
       <c r="K123" s="91" t="n"/>
       <c r="L123" s="92">
-        <f>IFERROR(AVERAGEIF(G123:K123,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G123:K123),"-")</f>
         <v/>
       </c>
       <c r="M123" s="93" t="n"/>
@@ -7787,7 +7708,7 @@
       <c r="J124" s="91" t="n"/>
       <c r="K124" s="91" t="n"/>
       <c r="L124" s="92">
-        <f>IFERROR(AVERAGEIF(G124:K124,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G124:K124),"-")</f>
         <v/>
       </c>
       <c r="M124" s="93" t="n"/>
@@ -7831,7 +7752,7 @@
       <c r="J125" s="91" t="n"/>
       <c r="K125" s="91" t="n"/>
       <c r="L125" s="92">
-        <f>IFERROR(AVERAGEIF(G125:K125,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G125:K125),"-")</f>
         <v/>
       </c>
       <c r="M125" s="93" t="n"/>
@@ -7875,7 +7796,7 @@
       <c r="J126" s="91" t="n"/>
       <c r="K126" s="91" t="n"/>
       <c r="L126" s="92">
-        <f>IFERROR(AVERAGEIF(G126:K126,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G126:K126),"-")</f>
         <v/>
       </c>
       <c r="M126" s="93" t="n"/>
@@ -7919,7 +7840,7 @@
       <c r="J127" s="91" t="n"/>
       <c r="K127" s="91" t="n"/>
       <c r="L127" s="92">
-        <f>IFERROR(AVERAGEIF(G127:K127,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G127:K127),"-")</f>
         <v/>
       </c>
       <c r="M127" s="93" t="n"/>
@@ -7963,7 +7884,7 @@
       <c r="J128" s="91" t="n"/>
       <c r="K128" s="91" t="n"/>
       <c r="L128" s="92">
-        <f>IFERROR(AVERAGEIF(G128:K128,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G128:K128),"-")</f>
         <v/>
       </c>
       <c r="M128" s="93" t="n"/>
@@ -8007,7 +7928,7 @@
       <c r="J129" s="91" t="n"/>
       <c r="K129" s="91" t="n"/>
       <c r="L129" s="92">
-        <f>IFERROR(AVERAGEIF(G129:K129,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G129:K129),"-")</f>
         <v/>
       </c>
       <c r="M129" s="93" t="n"/>
@@ -8051,7 +7972,7 @@
       <c r="J130" s="91" t="n"/>
       <c r="K130" s="91" t="n"/>
       <c r="L130" s="92">
-        <f>IFERROR(AVERAGEIF(G130:K130,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G130:K130),"-")</f>
         <v/>
       </c>
       <c r="M130" s="93" t="n"/>
@@ -8095,7 +8016,7 @@
       <c r="J131" s="91" t="n"/>
       <c r="K131" s="91" t="n"/>
       <c r="L131" s="92">
-        <f>IFERROR(AVERAGEIF(G131:K131,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G131:K131),"-")</f>
         <v/>
       </c>
       <c r="M131" s="93" t="n"/>
@@ -8139,7 +8060,7 @@
       <c r="J132" s="91" t="n"/>
       <c r="K132" s="91" t="n"/>
       <c r="L132" s="92">
-        <f>IFERROR(AVERAGEIF(G132:K132,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G132:K132),"-")</f>
         <v/>
       </c>
       <c r="M132" s="93" t="n"/>
@@ -8183,7 +8104,7 @@
       <c r="J133" s="91" t="n"/>
       <c r="K133" s="91" t="n"/>
       <c r="L133" s="92">
-        <f>IFERROR(AVERAGEIF(G133:K133,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G133:K133),"-")</f>
         <v/>
       </c>
       <c r="M133" s="93" t="n"/>
@@ -8227,7 +8148,7 @@
       <c r="J134" s="91" t="n"/>
       <c r="K134" s="91" t="n"/>
       <c r="L134" s="92">
-        <f>IFERROR(AVERAGEIF(G134:K134,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G134:K134),"-")</f>
         <v/>
       </c>
       <c r="M134" s="93" t="n"/>
@@ -8271,7 +8192,7 @@
       <c r="J135" s="91" t="n"/>
       <c r="K135" s="91" t="n"/>
       <c r="L135" s="92">
-        <f>IFERROR(AVERAGEIF(G135:K135,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G135:K135),"-")</f>
         <v/>
       </c>
       <c r="M135" s="93" t="n"/>
@@ -8315,7 +8236,7 @@
       <c r="J136" s="91" t="n"/>
       <c r="K136" s="91" t="n"/>
       <c r="L136" s="92">
-        <f>IFERROR(AVERAGEIF(G136:K136,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G136:K136),"-")</f>
         <v/>
       </c>
       <c r="M136" s="93" t="n"/>
@@ -8359,7 +8280,7 @@
       <c r="J137" s="91" t="n"/>
       <c r="K137" s="91" t="n"/>
       <c r="L137" s="92">
-        <f>IFERROR(AVERAGEIF(G137:K137,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G137:K137),"-")</f>
         <v/>
       </c>
       <c r="M137" s="93" t="n"/>
@@ -8403,7 +8324,7 @@
       <c r="J138" s="91" t="n"/>
       <c r="K138" s="91" t="n"/>
       <c r="L138" s="92">
-        <f>IFERROR(AVERAGEIF(G138:K138,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G138:K138),"-")</f>
         <v/>
       </c>
       <c r="M138" s="93" t="n"/>
@@ -8447,7 +8368,7 @@
       <c r="J139" s="91" t="n"/>
       <c r="K139" s="91" t="n"/>
       <c r="L139" s="92">
-        <f>IFERROR(AVERAGEIF(G139:K139,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G139:K139),"-")</f>
         <v/>
       </c>
       <c r="M139" s="93" t="n"/>
@@ -8491,7 +8412,7 @@
       <c r="J140" s="91" t="n"/>
       <c r="K140" s="91" t="n"/>
       <c r="L140" s="92">
-        <f>IFERROR(AVERAGEIF(G140:K140,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G140:K140),"-")</f>
         <v/>
       </c>
       <c r="M140" s="93" t="n"/>
@@ -8535,7 +8456,7 @@
       <c r="J141" s="91" t="n"/>
       <c r="K141" s="91" t="n"/>
       <c r="L141" s="92">
-        <f>IFERROR(AVERAGEIF(G141:K141,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G141:K141),"-")</f>
         <v/>
       </c>
       <c r="M141" s="93" t="n"/>
@@ -8579,7 +8500,7 @@
       <c r="J142" s="91" t="n"/>
       <c r="K142" s="91" t="n"/>
       <c r="L142" s="92">
-        <f>IFERROR(AVERAGEIF(G142:K142,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G142:K142),"-")</f>
         <v/>
       </c>
       <c r="M142" s="93" t="n"/>
@@ -8623,7 +8544,7 @@
       <c r="J143" s="91" t="n"/>
       <c r="K143" s="91" t="n"/>
       <c r="L143" s="92">
-        <f>IFERROR(AVERAGEIF(G143:K143,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G143:K143),"-")</f>
         <v/>
       </c>
       <c r="M143" s="93" t="n"/>
@@ -8667,7 +8588,7 @@
       <c r="J144" s="91" t="n"/>
       <c r="K144" s="91" t="n"/>
       <c r="L144" s="92">
-        <f>IFERROR(AVERAGEIF(G144:K144,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G144:K144),"-")</f>
         <v/>
       </c>
       <c r="M144" s="93" t="n"/>
@@ -8711,7 +8632,7 @@
       <c r="J145" s="91" t="n"/>
       <c r="K145" s="91" t="n"/>
       <c r="L145" s="92">
-        <f>IFERROR(AVERAGEIF(G145:K145,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G145:K145),"-")</f>
         <v/>
       </c>
       <c r="M145" s="93" t="n"/>
@@ -8755,7 +8676,7 @@
       <c r="J146" s="91" t="n"/>
       <c r="K146" s="91" t="n"/>
       <c r="L146" s="92">
-        <f>IFERROR(AVERAGEIF(G146:K146,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G146:K146),"-")</f>
         <v/>
       </c>
       <c r="M146" s="93" t="n"/>
@@ -8799,7 +8720,7 @@
       <c r="J147" s="91" t="n"/>
       <c r="K147" s="91" t="n"/>
       <c r="L147" s="92">
-        <f>IFERROR(AVERAGEIF(G147:K147,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G147:K147),"-")</f>
         <v/>
       </c>
       <c r="M147" s="93" t="n"/>
@@ -8847,7 +8768,7 @@
       <c r="J148" s="91" t="n"/>
       <c r="K148" s="91" t="n"/>
       <c r="L148" s="92">
-        <f>IFERROR(AVERAGEIF(G148:K148,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G148:K148),"-")</f>
         <v/>
       </c>
       <c r="M148" s="93" t="inlineStr">
@@ -8903,7 +8824,7 @@
       <c r="J149" s="91" t="n"/>
       <c r="K149" s="91" t="n"/>
       <c r="L149" s="92">
-        <f>IFERROR(AVERAGEIF(G149:K149,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G149:K149),"-")</f>
         <v/>
       </c>
       <c r="M149" s="93" t="inlineStr">
@@ -8959,7 +8880,7 @@
       <c r="J150" s="91" t="n"/>
       <c r="K150" s="91" t="n"/>
       <c r="L150" s="92">
-        <f>IFERROR(AVERAGEIF(G150:K150,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G150:K150),"-")</f>
         <v/>
       </c>
       <c r="M150" s="93" t="inlineStr">
@@ -9015,7 +8936,7 @@
       <c r="J151" s="91" t="n"/>
       <c r="K151" s="91" t="n"/>
       <c r="L151" s="92">
-        <f>IFERROR(AVERAGEIF(G151:K151,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G151:K151),"-")</f>
         <v/>
       </c>
       <c r="M151" s="93" t="inlineStr">
@@ -9071,7 +8992,7 @@
       <c r="J152" s="91" t="n"/>
       <c r="K152" s="91" t="n"/>
       <c r="L152" s="92">
-        <f>IFERROR(AVERAGEIF(G152:K152,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G152:K152),"-")</f>
         <v/>
       </c>
       <c r="M152" s="93" t="inlineStr">
@@ -9127,7 +9048,7 @@
       <c r="J153" s="91" t="n"/>
       <c r="K153" s="91" t="n"/>
       <c r="L153" s="92">
-        <f>IFERROR(AVERAGEIF(G153:K153,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G153:K153),"-")</f>
         <v/>
       </c>
       <c r="M153" s="93" t="inlineStr">
@@ -9185,7 +9106,7 @@
       <c r="J154" s="91" t="n"/>
       <c r="K154" s="91" t="n"/>
       <c r="L154" s="92">
-        <f>IFERROR(AVERAGEIF(G154:K154,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G154:K154),"-")</f>
         <v/>
       </c>
       <c r="M154" s="93" t="inlineStr">
@@ -9249,7 +9170,7 @@
       </c>
       <c r="K155" s="91" t="n"/>
       <c r="L155" s="92">
-        <f>IFERROR(AVERAGEIF(G155:K155,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G155:K155),"-")</f>
         <v/>
       </c>
       <c r="M155" s="93" t="inlineStr">
@@ -9317,7 +9238,7 @@
       </c>
       <c r="K156" s="91" t="n"/>
       <c r="L156" s="92">
-        <f>IFERROR(AVERAGEIF(G156:K156,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G156:K156),"-")</f>
         <v/>
       </c>
       <c r="M156" s="93" t="inlineStr">
@@ -9385,7 +9306,7 @@
       </c>
       <c r="K157" s="91" t="n"/>
       <c r="L157" s="92">
-        <f>IFERROR(AVERAGEIF(G157:K157,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G157:K157),"-")</f>
         <v/>
       </c>
       <c r="M157" s="93" t="inlineStr">
@@ -9453,7 +9374,7 @@
       </c>
       <c r="K158" s="91" t="n"/>
       <c r="L158" s="92">
-        <f>IFERROR(AVERAGEIF(G158:K158,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G158:K158),"-")</f>
         <v/>
       </c>
       <c r="M158" s="93" t="inlineStr">
@@ -9521,7 +9442,7 @@
       </c>
       <c r="K159" s="91" t="n"/>
       <c r="L159" s="92">
-        <f>IFERROR(AVERAGEIF(G159:K159,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G159:K159),"-")</f>
         <v/>
       </c>
       <c r="M159" s="93" t="inlineStr">
@@ -9589,7 +9510,7 @@
       </c>
       <c r="K160" s="91" t="n"/>
       <c r="L160" s="92">
-        <f>IFERROR(AVERAGEIF(G160:K160,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G160:K160),"-")</f>
         <v/>
       </c>
       <c r="M160" s="93" t="inlineStr">
@@ -9651,7 +9572,7 @@
       <c r="J161" s="91" t="n"/>
       <c r="K161" s="91" t="n"/>
       <c r="L161" s="92">
-        <f>IFERROR(AVERAGEIF(G161:K161,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G161:K161),"-")</f>
         <v/>
       </c>
       <c r="M161" s="93" t="inlineStr">
@@ -9701,7 +9622,7 @@
       <c r="J162" s="91" t="n"/>
       <c r="K162" s="91" t="n"/>
       <c r="L162" s="92">
-        <f>IFERROR(AVERAGEIF(G162:K162,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G162:K162),"-")</f>
         <v/>
       </c>
       <c r="M162" s="93" t="inlineStr">
@@ -9752,7 +9673,7 @@
       <c r="J163" s="91" t="n"/>
       <c r="K163" s="91" t="n"/>
       <c r="L163" s="92">
-        <f>IFERROR(AVERAGEIF(G163:K163,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G163:K163),"-")</f>
         <v/>
       </c>
       <c r="M163" s="93" t="inlineStr">
@@ -9800,7 +9721,7 @@
       <c r="J164" s="91" t="n"/>
       <c r="K164" s="91" t="n"/>
       <c r="L164" s="92">
-        <f>IFERROR(AVERAGEIF(G164:K164,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G164:K164),"-")</f>
         <v/>
       </c>
       <c r="M164" s="93" t="n"/>
@@ -9844,7 +9765,7 @@
       <c r="J165" s="91" t="n"/>
       <c r="K165" s="91" t="n"/>
       <c r="L165" s="92">
-        <f>IFERROR(AVERAGEIF(G165:K165,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G165:K165),"-")</f>
         <v/>
       </c>
       <c r="M165" s="93" t="n"/>
@@ -9888,7 +9809,7 @@
       <c r="J166" s="91" t="n"/>
       <c r="K166" s="91" t="n"/>
       <c r="L166" s="92">
-        <f>IFERROR(AVERAGEIF(G166:K166,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G166:K166),"-")</f>
         <v/>
       </c>
       <c r="M166" s="93" t="n"/>
@@ -9932,7 +9853,7 @@
       <c r="J167" s="91" t="n"/>
       <c r="K167" s="91" t="n"/>
       <c r="L167" s="92">
-        <f>IFERROR(AVERAGEIF(G167:K167,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G167:K167),"-")</f>
         <v/>
       </c>
       <c r="M167" s="93" t="n"/>
@@ -9950,7 +9871,7 @@
       </c>
       <c r="T167" t="inlineStr">
         <is>
-          <t>BORU</t>
+          <t>FİTTİNG</t>
         </is>
       </c>
     </row>
@@ -9976,7 +9897,7 @@
       <c r="J168" s="91" t="n"/>
       <c r="K168" s="91" t="n"/>
       <c r="L168" s="92">
-        <f>IFERROR(AVERAGEIF(G168:K168,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G168:K168),"-")</f>
         <v/>
       </c>
       <c r="M168" s="93" t="n"/>
@@ -9994,7 +9915,7 @@
       </c>
       <c r="T168" t="inlineStr">
         <is>
-          <t>BORU</t>
+          <t>FİTTİNG</t>
         </is>
       </c>
     </row>
@@ -10020,7 +9941,7 @@
       <c r="J169" s="91" t="n"/>
       <c r="K169" s="91" t="n"/>
       <c r="L169" s="92">
-        <f>IFERROR(AVERAGEIF(G169:K169,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G169:K169),"-")</f>
         <v/>
       </c>
       <c r="M169" s="93" t="n"/>
@@ -10038,7 +9959,7 @@
       </c>
       <c r="T169" t="inlineStr">
         <is>
-          <t>BORU</t>
+          <t>FİTTİNG</t>
         </is>
       </c>
     </row>
@@ -10064,7 +9985,7 @@
       <c r="J170" s="91" t="n"/>
       <c r="K170" s="91" t="n"/>
       <c r="L170" s="92">
-        <f>IFERROR(AVERAGEIF(G170:K170,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G170:K170),"-")</f>
         <v/>
       </c>
       <c r="M170" s="93" t="n"/>
@@ -10108,7 +10029,7 @@
       <c r="J171" s="91" t="n"/>
       <c r="K171" s="91" t="n"/>
       <c r="L171" s="92">
-        <f>IFERROR(AVERAGEIF(G171:K171,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G171:K171),"-")</f>
         <v/>
       </c>
       <c r="M171" s="93" t="n"/>
@@ -10152,7 +10073,7 @@
       <c r="J172" s="91" t="n"/>
       <c r="K172" s="91" t="n"/>
       <c r="L172" s="92">
-        <f>IFERROR(AVERAGEIF(G172:K172,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G172:K172),"-")</f>
         <v/>
       </c>
       <c r="M172" s="93" t="n"/>
@@ -10196,7 +10117,7 @@
       <c r="J173" s="91" t="n"/>
       <c r="K173" s="91" t="n"/>
       <c r="L173" s="92">
-        <f>IFERROR(AVERAGEIF(G173:K173,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G173:K173),"-")</f>
         <v/>
       </c>
       <c r="M173" s="93" t="n"/>
@@ -10240,7 +10161,7 @@
       <c r="J174" s="91" t="n"/>
       <c r="K174" s="91" t="n"/>
       <c r="L174" s="92">
-        <f>IFERROR(AVERAGEIF(G174:K174,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G174:K174),"-")</f>
         <v/>
       </c>
       <c r="M174" s="93" t="n"/>
@@ -10288,7 +10209,7 @@
       <c r="J175" s="91" t="n"/>
       <c r="K175" s="91" t="n"/>
       <c r="L175" s="92">
-        <f>IFERROR(AVERAGEIF(G175:K175,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G175:K175),"-")</f>
         <v/>
       </c>
       <c r="M175" s="93" t="inlineStr">
@@ -10312,11 +10233,6 @@
         <f>IFERROR(INDEX(M175:Q175,MATCH(MIN(G175:K175),G175:K175,0)),"-")</f>
         <v/>
       </c>
-      <c r="T175" t="inlineStr">
-        <is>
-          <t>VANA</t>
-        </is>
-      </c>
     </row>
     <row r="176" ht="24" customHeight="1">
       <c r="A176" s="90" t="n">
@@ -10344,7 +10260,7 @@
       <c r="J176" s="91" t="n"/>
       <c r="K176" s="91" t="n"/>
       <c r="L176" s="92">
-        <f>IFERROR(AVERAGEIF(G176:K176,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G176:K176),"-")</f>
         <v/>
       </c>
       <c r="M176" s="93" t="inlineStr">
@@ -10368,11 +10284,6 @@
         <f>IFERROR(INDEX(M176:Q176,MATCH(MIN(G176:K176),G176:K176,0)),"-")</f>
         <v/>
       </c>
-      <c r="T176" t="inlineStr">
-        <is>
-          <t>VANA</t>
-        </is>
-      </c>
     </row>
     <row r="177" ht="24" customHeight="1">
       <c r="A177" s="90" t="n">
@@ -10383,22 +10294,56 @@
           <t>OZEL-168</t>
         </is>
       </c>
-      <c r="D177" s="61" t="n"/>
-      <c r="E177" s="60" t="n"/>
-      <c r="F177" s="60" t="n"/>
-      <c r="G177" s="91" t="n"/>
-      <c r="H177" s="91" t="n"/>
-      <c r="I177" s="91" t="n"/>
-      <c r="J177" s="91" t="n"/>
+      <c r="D177" s="61" t="inlineStr">
+        <is>
+          <t>1/2", Ball Valve, Reduced Bore, ASTM A105, 800# Threaded</t>
+        </is>
+      </c>
+      <c r="E177" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F177" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G177" s="96" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="H177" s="97" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="I177" s="97" t="n">
+        <v>66</v>
+      </c>
+      <c r="J177" s="97" t="n">
+        <v>315</v>
+      </c>
       <c r="K177" s="91" t="n"/>
       <c r="L177" s="92">
-        <f>IFERROR(AVERAGEIF(G177:K177,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M177" s="93" t="n"/>
-      <c r="N177" s="93" t="n"/>
-      <c r="O177" s="93" t="n"/>
-      <c r="P177" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G177:K177),"-")</f>
+        <v/>
+      </c>
+      <c r="M177" s="93" t="inlineStr">
+        <is>
+          <t>VALFTEK</t>
+        </is>
+      </c>
+      <c r="N177" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="O177" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="P177" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="Q177" s="93" t="n"/>
       <c r="R177" s="92">
         <f>IFERROR(MIN(G177:K177),"-")</f>
@@ -10408,7 +10353,11 @@
         <f>IFERROR(INDEX(M177:Q177,MATCH(MIN(G177:K177),G177:K177,0)),"-")</f>
         <v/>
       </c>
-      <c r="T177" t="inlineStr"/>
+      <c r="T177" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="178" ht="24" customHeight="1">
       <c r="A178" s="90" t="n">
@@ -10419,22 +10368,56 @@
           <t>OZEL-169</t>
         </is>
       </c>
-      <c r="D178" s="61" t="n"/>
-      <c r="E178" s="60" t="n"/>
-      <c r="F178" s="60" t="n"/>
-      <c r="G178" s="91" t="n"/>
-      <c r="H178" s="91" t="n"/>
-      <c r="I178" s="91" t="n"/>
-      <c r="J178" s="91" t="n"/>
+      <c r="D178" s="61" t="inlineStr">
+        <is>
+          <t>2", Ball Valve, Reduced Bore, ASTM A105, 800# Threaded</t>
+        </is>
+      </c>
+      <c r="E178" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F178" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G178" s="96" t="n">
+        <v>240.8</v>
+      </c>
+      <c r="H178" s="97" t="n">
+        <v>252.8</v>
+      </c>
+      <c r="I178" s="97" t="n">
+        <v>270</v>
+      </c>
+      <c r="J178" s="97" t="n">
+        <v>801</v>
+      </c>
       <c r="K178" s="91" t="n"/>
       <c r="L178" s="92">
-        <f>IFERROR(AVERAGEIF(G178:K178,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M178" s="93" t="n"/>
-      <c r="N178" s="93" t="n"/>
-      <c r="O178" s="93" t="n"/>
-      <c r="P178" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G178:K178),"-")</f>
+        <v/>
+      </c>
+      <c r="M178" s="93" t="inlineStr">
+        <is>
+          <t>VALFTEK</t>
+        </is>
+      </c>
+      <c r="N178" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="O178" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="P178" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="Q178" s="93" t="n"/>
       <c r="R178" s="92">
         <f>IFERROR(MIN(G178:K178),"-")</f>
@@ -10444,7 +10427,11 @@
         <f>IFERROR(INDEX(M178:Q178,MATCH(MIN(G178:K178),G178:K178,0)),"-")</f>
         <v/>
       </c>
-      <c r="T178" t="inlineStr"/>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="179" ht="24" customHeight="1">
       <c r="A179" s="90" t="n">
@@ -10455,22 +10442,56 @@
           <t>OZEL-170</t>
         </is>
       </c>
-      <c r="D179" s="61" t="n"/>
-      <c r="E179" s="60" t="n"/>
-      <c r="F179" s="60" t="n"/>
-      <c r="G179" s="91" t="n"/>
-      <c r="H179" s="91" t="n"/>
-      <c r="I179" s="91" t="n"/>
-      <c r="J179" s="91" t="n"/>
+      <c r="D179" s="61" t="inlineStr">
+        <is>
+          <t>3/4", Ball Valve, Reduced Bore, ASTM A105, 800# Threaded</t>
+        </is>
+      </c>
+      <c r="E179" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F179" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G179" s="96" t="n">
+        <v>77</v>
+      </c>
+      <c r="H179" s="97" t="n">
+        <v>80</v>
+      </c>
+      <c r="I179" s="97" t="n">
+        <v>83</v>
+      </c>
+      <c r="J179" s="97" t="n">
+        <v>321</v>
+      </c>
       <c r="K179" s="91" t="n"/>
       <c r="L179" s="92">
-        <f>IFERROR(AVERAGEIF(G179:K179,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M179" s="93" t="n"/>
-      <c r="N179" s="93" t="n"/>
-      <c r="O179" s="93" t="n"/>
-      <c r="P179" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G179:K179),"-")</f>
+        <v/>
+      </c>
+      <c r="M179" s="93" t="inlineStr">
+        <is>
+          <t>VALFTEK</t>
+        </is>
+      </c>
+      <c r="N179" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="O179" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="P179" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="Q179" s="93" t="n"/>
       <c r="R179" s="92">
         <f>IFERROR(MIN(G179:K179),"-")</f>
@@ -10480,7 +10501,11 @@
         <f>IFERROR(INDEX(M179:Q179,MATCH(MIN(G179:K179),G179:K179,0)),"-")</f>
         <v/>
       </c>
-      <c r="T179" t="inlineStr"/>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="180" ht="24" customHeight="1">
       <c r="A180" s="90" t="n">
@@ -10491,22 +10516,56 @@
           <t>OZEL-171</t>
         </is>
       </c>
-      <c r="D180" s="61" t="n"/>
-      <c r="E180" s="60" t="n"/>
-      <c r="F180" s="60" t="n"/>
-      <c r="G180" s="91" t="n"/>
-      <c r="H180" s="91" t="n"/>
-      <c r="I180" s="91" t="n"/>
-      <c r="J180" s="91" t="n"/>
+      <c r="D180" s="61" t="inlineStr">
+        <is>
+          <t>1/2", Ball Valve, Reduced Bore, ASTM A105, 800# Threaded</t>
+        </is>
+      </c>
+      <c r="E180" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F180" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G180" s="96" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="H180" s="97" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="I180" s="97" t="n">
+        <v>66</v>
+      </c>
+      <c r="J180" s="97" t="n">
+        <v>315</v>
+      </c>
       <c r="K180" s="91" t="n"/>
       <c r="L180" s="92">
-        <f>IFERROR(AVERAGEIF(G180:K180,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M180" s="93" t="n"/>
-      <c r="N180" s="93" t="n"/>
-      <c r="O180" s="93" t="n"/>
-      <c r="P180" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G180:K180),"-")</f>
+        <v/>
+      </c>
+      <c r="M180" s="93" t="inlineStr">
+        <is>
+          <t>VALFTEK</t>
+        </is>
+      </c>
+      <c r="N180" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="O180" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="P180" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="Q180" s="93" t="n"/>
       <c r="R180" s="92">
         <f>IFERROR(MIN(G180:K180),"-")</f>
@@ -10516,7 +10575,11 @@
         <f>IFERROR(INDEX(M180:Q180,MATCH(MIN(G180:K180),G180:K180,0)),"-")</f>
         <v/>
       </c>
-      <c r="T180" t="inlineStr"/>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="24" customHeight="1">
       <c r="A181" s="90" t="n"/>
@@ -10525,26 +10588,70 @@
           <t>OZEL-172</t>
         </is>
       </c>
-      <c r="D181" s="21" t="n"/>
-      <c r="E181" s="60" t="n"/>
-      <c r="F181" s="60" t="n"/>
-      <c r="G181" s="91" t="n"/>
-      <c r="H181" s="91" t="n"/>
-      <c r="I181" s="91" t="n"/>
-      <c r="J181" s="91" t="n"/>
+      <c r="D181" s="21" t="inlineStr">
+        <is>
+          <t>1/2", Ball Valve, Reduced Bore, ASTM A105, 800# Threaded</t>
+        </is>
+      </c>
+      <c r="E181" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F181" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="G181" s="96" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="H181" s="97" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="I181" s="97" t="n">
+        <v>66</v>
+      </c>
+      <c r="J181" s="97" t="n">
+        <v>315</v>
+      </c>
       <c r="K181" s="91" t="n"/>
-      <c r="L181" s="92" t="n"/>
-      <c r="M181" s="93" t="n"/>
-      <c r="N181" s="93" t="n"/>
-      <c r="O181" s="93" t="n"/>
-      <c r="P181" s="93" t="n"/>
+      <c r="L181" s="92">
+        <f>IFERROR(AVERAGE(G181:K181),"-")</f>
+        <v/>
+      </c>
+      <c r="M181" s="93" t="inlineStr">
+        <is>
+          <t>VALFTEK</t>
+        </is>
+      </c>
+      <c r="N181" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="O181" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="P181" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="Q181" s="93" t="n"/>
-      <c r="R181" s="92" t="n"/>
+      <c r="R181" s="92">
+        <f>IFERROR(MIN(G181:K181),"-")</f>
+        <v/>
+      </c>
       <c r="S181" s="9">
         <f>IFERROR(INDEX(M181:Q181,MATCH(MIN(G181:K181),G181:K181,0)),"-")</f>
         <v/>
       </c>
-      <c r="T181" t="inlineStr"/>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="24" customHeight="1">
       <c r="A182" s="90" t="n"/>
@@ -10553,26 +10660,70 @@
           <t>OZEL-173</t>
         </is>
       </c>
-      <c r="D182" s="21" t="n"/>
-      <c r="E182" s="60" t="n"/>
-      <c r="F182" s="60" t="n"/>
-      <c r="G182" s="91" t="n"/>
-      <c r="H182" s="91" t="n"/>
-      <c r="I182" s="91" t="n"/>
-      <c r="J182" s="91" t="n"/>
+      <c r="D182" s="21" t="inlineStr">
+        <is>
+          <t>3/4", Ball Valve, Reduced Bore, ASTM A105, 800# Threaded</t>
+        </is>
+      </c>
+      <c r="E182" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F182" s="60" t="n">
+        <v>6</v>
+      </c>
+      <c r="G182" s="96" t="n">
+        <v>77</v>
+      </c>
+      <c r="H182" s="97" t="n">
+        <v>80</v>
+      </c>
+      <c r="I182" s="97" t="n">
+        <v>83</v>
+      </c>
+      <c r="J182" s="97" t="n">
+        <v>321</v>
+      </c>
       <c r="K182" s="91" t="n"/>
-      <c r="L182" s="92" t="n"/>
-      <c r="M182" s="93" t="n"/>
-      <c r="N182" s="93" t="n"/>
-      <c r="O182" s="93" t="n"/>
-      <c r="P182" s="93" t="n"/>
+      <c r="L182" s="92">
+        <f>IFERROR(AVERAGE(G182:K182),"-")</f>
+        <v/>
+      </c>
+      <c r="M182" s="93" t="inlineStr">
+        <is>
+          <t>VALFTEK</t>
+        </is>
+      </c>
+      <c r="N182" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="O182" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="P182" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="Q182" s="93" t="n"/>
-      <c r="R182" s="92" t="n"/>
+      <c r="R182" s="92">
+        <f>IFERROR(MIN(G182:K182),"-")</f>
+        <v/>
+      </c>
       <c r="S182" s="9">
         <f>IFERROR(INDEX(M182:Q182,MATCH(MIN(G182:K182),G182:K182,0)),"-")</f>
         <v/>
       </c>
-      <c r="T182" t="inlineStr"/>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="24" customHeight="1">
       <c r="A183" s="90" t="n"/>
@@ -10581,26 +10732,70 @@
           <t>OZEL-174</t>
         </is>
       </c>
-      <c r="D183" s="21" t="n"/>
-      <c r="E183" s="60" t="n"/>
-      <c r="F183" s="60" t="n"/>
-      <c r="G183" s="91" t="n"/>
-      <c r="H183" s="91" t="n"/>
-      <c r="I183" s="91" t="n"/>
-      <c r="J183" s="91" t="n"/>
+      <c r="D183" s="21" t="inlineStr">
+        <is>
+          <t>1/2", Ball Valve, Reduced Bore, ASTM A105, 800# Threaded</t>
+        </is>
+      </c>
+      <c r="E183" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F183" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="G183" s="96" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="H183" s="97" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="I183" s="97" t="n">
+        <v>66</v>
+      </c>
+      <c r="J183" s="97" t="n">
+        <v>315</v>
+      </c>
       <c r="K183" s="91" t="n"/>
-      <c r="L183" s="92" t="n"/>
-      <c r="M183" s="93" t="n"/>
-      <c r="N183" s="93" t="n"/>
-      <c r="O183" s="93" t="n"/>
-      <c r="P183" s="93" t="n"/>
+      <c r="L183" s="92">
+        <f>IFERROR(AVERAGE(G183:K183),"-")</f>
+        <v/>
+      </c>
+      <c r="M183" s="93" t="inlineStr">
+        <is>
+          <t>VALFTEK</t>
+        </is>
+      </c>
+      <c r="N183" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="O183" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="P183" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="Q183" s="93" t="n"/>
-      <c r="R183" s="92" t="n"/>
+      <c r="R183" s="92">
+        <f>IFERROR(MIN(G183:K183),"-")</f>
+        <v/>
+      </c>
       <c r="S183" s="9">
         <f>IFERROR(INDEX(M183:Q183,MATCH(MIN(G183:K183),G183:K183,0)),"-")</f>
         <v/>
       </c>
-      <c r="T183" t="inlineStr"/>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="24" customHeight="1">
       <c r="A184" s="90" t="n"/>
@@ -10609,26 +10804,70 @@
           <t>OZEL-175</t>
         </is>
       </c>
-      <c r="D184" s="21" t="n"/>
-      <c r="E184" s="60" t="n"/>
-      <c r="F184" s="60" t="n"/>
-      <c r="G184" s="91" t="n"/>
-      <c r="H184" s="91" t="n"/>
-      <c r="I184" s="91" t="n"/>
-      <c r="J184" s="91" t="n"/>
+      <c r="D184" s="21" t="inlineStr">
+        <is>
+          <t>3/4", Ball Valve, Reduced Bore, ASTM A105, 800# Threaded</t>
+        </is>
+      </c>
+      <c r="E184" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F184" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G184" s="96" t="n">
+        <v>77</v>
+      </c>
+      <c r="H184" s="97" t="n">
+        <v>80</v>
+      </c>
+      <c r="I184" s="97" t="n">
+        <v>83</v>
+      </c>
+      <c r="J184" s="97" t="n">
+        <v>321</v>
+      </c>
       <c r="K184" s="91" t="n"/>
-      <c r="L184" s="92" t="n"/>
-      <c r="M184" s="93" t="n"/>
-      <c r="N184" s="93" t="n"/>
-      <c r="O184" s="93" t="n"/>
-      <c r="P184" s="93" t="n"/>
+      <c r="L184" s="92">
+        <f>IFERROR(AVERAGE(G184:K184),"-")</f>
+        <v/>
+      </c>
+      <c r="M184" s="93" t="inlineStr">
+        <is>
+          <t>VALFTEK</t>
+        </is>
+      </c>
+      <c r="N184" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="O184" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="P184" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="Q184" s="93" t="n"/>
-      <c r="R184" s="92" t="n"/>
+      <c r="R184" s="92">
+        <f>IFERROR(MIN(G184:K184),"-")</f>
+        <v/>
+      </c>
       <c r="S184" s="9">
         <f>IFERROR(INDEX(M184:Q184,MATCH(MIN(G184:K184),G184:K184,0)),"-")</f>
         <v/>
       </c>
-      <c r="T184" t="inlineStr"/>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="24" customHeight="1">
       <c r="A185" s="90" t="n"/>
@@ -10637,26 +10876,64 @@
           <t>OZEL-176</t>
         </is>
       </c>
-      <c r="D185" s="21" t="n"/>
-      <c r="E185" s="60" t="n"/>
-      <c r="F185" s="60" t="n"/>
-      <c r="G185" s="91" t="n"/>
-      <c r="H185" s="91" t="n"/>
-      <c r="I185" s="91" t="n"/>
+      <c r="D185" s="21" t="inlineStr">
+        <is>
+          <t>12", Gate Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E185" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F185" s="60" t="n">
+        <v>6</v>
+      </c>
+      <c r="G185" s="97" t="n">
+        <v>2799</v>
+      </c>
+      <c r="H185" s="97" t="n">
+        <v>2419</v>
+      </c>
+      <c r="I185" s="97" t="n">
+        <v>4600</v>
+      </c>
       <c r="J185" s="91" t="n"/>
       <c r="K185" s="91" t="n"/>
-      <c r="L185" s="92" t="n"/>
-      <c r="M185" s="93" t="n"/>
-      <c r="N185" s="93" t="n"/>
-      <c r="O185" s="93" t="n"/>
+      <c r="L185" s="92">
+        <f>IFERROR(AVERAGE(G185:K185),"-")</f>
+        <v/>
+      </c>
+      <c r="M185" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N185" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O185" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P185" s="93" t="n"/>
       <c r="Q185" s="93" t="n"/>
-      <c r="R185" s="92" t="n"/>
+      <c r="R185" s="92">
+        <f>IFERROR(MIN(G185:K185),"-")</f>
+        <v/>
+      </c>
       <c r="S185" s="9">
         <f>IFERROR(INDEX(M185:Q185,MATCH(MIN(G185:K185),G185:K185,0)),"-")</f>
         <v/>
       </c>
-      <c r="T185" t="inlineStr"/>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="186" ht="24" customHeight="1">
       <c r="A186" s="90" t="n"/>
@@ -10665,26 +10942,64 @@
           <t>OZEL-177</t>
         </is>
       </c>
-      <c r="D186" s="21" t="n"/>
-      <c r="E186" s="60" t="n"/>
-      <c r="F186" s="60" t="n"/>
-      <c r="G186" s="91" t="n"/>
-      <c r="H186" s="91" t="n"/>
-      <c r="I186" s="91" t="n"/>
+      <c r="D186" s="21" t="inlineStr">
+        <is>
+          <t>3", Gate Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E186" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F186" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="G186" s="97" t="n">
+        <v>380.7</v>
+      </c>
+      <c r="H186" s="97" t="n">
+        <v>340</v>
+      </c>
+      <c r="I186" s="97" t="n">
+        <v>644</v>
+      </c>
       <c r="J186" s="91" t="n"/>
       <c r="K186" s="91" t="n"/>
-      <c r="L186" s="92" t="n"/>
-      <c r="M186" s="93" t="n"/>
-      <c r="N186" s="93" t="n"/>
-      <c r="O186" s="93" t="n"/>
+      <c r="L186" s="92">
+        <f>IFERROR(AVERAGE(G186:K186),"-")</f>
+        <v/>
+      </c>
+      <c r="M186" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N186" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O186" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P186" s="93" t="n"/>
       <c r="Q186" s="93" t="n"/>
-      <c r="R186" s="92" t="n"/>
+      <c r="R186" s="92">
+        <f>IFERROR(MIN(G186:K186),"-")</f>
+        <v/>
+      </c>
       <c r="S186" s="9">
         <f>IFERROR(INDEX(M186:Q186,MATCH(MIN(G186:K186),G186:K186,0)),"-")</f>
         <v/>
       </c>
-      <c r="T186" t="inlineStr"/>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="187" ht="24" customHeight="1">
       <c r="A187" s="90" t="n"/>
@@ -10693,26 +11008,64 @@
           <t>OZEL-178</t>
         </is>
       </c>
-      <c r="D187" s="21" t="n"/>
-      <c r="E187" s="60" t="n"/>
-      <c r="F187" s="60" t="n"/>
-      <c r="G187" s="91" t="n"/>
-      <c r="H187" s="91" t="n"/>
-      <c r="I187" s="91" t="n"/>
+      <c r="D187" s="21" t="inlineStr">
+        <is>
+          <t>4", Gate Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E187" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F187" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G187" s="97" t="n">
+        <v>490.05</v>
+      </c>
+      <c r="H187" s="97" t="n">
+        <v>478</v>
+      </c>
+      <c r="I187" s="97" t="n">
+        <v>992</v>
+      </c>
       <c r="J187" s="91" t="n"/>
       <c r="K187" s="91" t="n"/>
-      <c r="L187" s="92" t="n"/>
-      <c r="M187" s="93" t="n"/>
-      <c r="N187" s="93" t="n"/>
-      <c r="O187" s="93" t="n"/>
+      <c r="L187" s="92">
+        <f>IFERROR(AVERAGE(G187:K187),"-")</f>
+        <v/>
+      </c>
+      <c r="M187" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N187" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O187" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P187" s="93" t="n"/>
       <c r="Q187" s="93" t="n"/>
-      <c r="R187" s="92" t="n"/>
+      <c r="R187" s="92">
+        <f>IFERROR(MIN(G187:K187),"-")</f>
+        <v/>
+      </c>
       <c r="S187" s="9">
         <f>IFERROR(INDEX(M187:Q187,MATCH(MIN(G187:K187),G187:K187,0)),"-")</f>
         <v/>
       </c>
-      <c r="T187" t="inlineStr"/>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="188" ht="24" customHeight="1">
       <c r="A188" s="90" t="n"/>
@@ -10721,26 +11074,64 @@
           <t>OZEL-179</t>
         </is>
       </c>
-      <c r="D188" s="21" t="n"/>
-      <c r="E188" s="60" t="n"/>
-      <c r="F188" s="60" t="n"/>
-      <c r="G188" s="91" t="n"/>
-      <c r="H188" s="91" t="n"/>
-      <c r="I188" s="91" t="n"/>
+      <c r="D188" s="21" t="inlineStr">
+        <is>
+          <t>6", Gate Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E188" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F188" s="60" t="n">
+        <v>6</v>
+      </c>
+      <c r="G188" s="97" t="n">
+        <v>789.75</v>
+      </c>
+      <c r="H188" s="97" t="n">
+        <v>757</v>
+      </c>
+      <c r="I188" s="97" t="n">
+        <v>1564</v>
+      </c>
       <c r="J188" s="91" t="n"/>
       <c r="K188" s="91" t="n"/>
-      <c r="L188" s="92" t="n"/>
-      <c r="M188" s="93" t="n"/>
-      <c r="N188" s="93" t="n"/>
-      <c r="O188" s="93" t="n"/>
+      <c r="L188" s="92">
+        <f>IFERROR(AVERAGE(G188:K188),"-")</f>
+        <v/>
+      </c>
+      <c r="M188" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N188" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O188" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P188" s="93" t="n"/>
       <c r="Q188" s="93" t="n"/>
-      <c r="R188" s="92" t="n"/>
+      <c r="R188" s="92">
+        <f>IFERROR(MIN(G188:K188),"-")</f>
+        <v/>
+      </c>
       <c r="S188" s="9">
         <f>IFERROR(INDEX(M188:Q188,MATCH(MIN(G188:K188),G188:K188,0)),"-")</f>
         <v/>
       </c>
-      <c r="T188" t="inlineStr"/>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="189" ht="24" customHeight="1">
       <c r="A189" s="90" t="n"/>
@@ -10749,26 +11140,64 @@
           <t>OZEL-180</t>
         </is>
       </c>
-      <c r="D189" s="21" t="n"/>
-      <c r="E189" s="60" t="n"/>
-      <c r="F189" s="60" t="n"/>
-      <c r="G189" s="91" t="n"/>
-      <c r="H189" s="91" t="n"/>
-      <c r="I189" s="91" t="n"/>
+      <c r="D189" s="21" t="inlineStr">
+        <is>
+          <t>8", Gate Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E189" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F189" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G189" s="97" t="n">
+        <v>1283.85</v>
+      </c>
+      <c r="H189" s="97" t="n">
+        <v>1104</v>
+      </c>
+      <c r="I189" s="97" t="n">
+        <v>2124</v>
+      </c>
       <c r="J189" s="91" t="n"/>
       <c r="K189" s="91" t="n"/>
-      <c r="L189" s="92" t="n"/>
-      <c r="M189" s="93" t="n"/>
-      <c r="N189" s="93" t="n"/>
-      <c r="O189" s="93" t="n"/>
+      <c r="L189" s="92">
+        <f>IFERROR(AVERAGE(G189:K189),"-")</f>
+        <v/>
+      </c>
+      <c r="M189" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N189" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O189" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P189" s="93" t="n"/>
       <c r="Q189" s="93" t="n"/>
-      <c r="R189" s="92" t="n"/>
+      <c r="R189" s="92">
+        <f>IFERROR(MIN(G189:K189),"-")</f>
+        <v/>
+      </c>
       <c r="S189" s="9">
         <f>IFERROR(INDEX(M189:Q189,MATCH(MIN(G189:K189),G189:K189,0)),"-")</f>
         <v/>
       </c>
-      <c r="T189" t="inlineStr"/>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="190" ht="24" customHeight="1">
       <c r="A190" s="90" t="n">
@@ -10779,21 +11208,49 @@
           <t>OZEL-181</t>
         </is>
       </c>
-      <c r="D190" s="21" t="n"/>
-      <c r="E190" s="60" t="n"/>
-      <c r="F190" s="60" t="n"/>
-      <c r="G190" s="91" t="n"/>
-      <c r="H190" s="91" t="n"/>
-      <c r="I190" s="91" t="n"/>
+      <c r="D190" s="21" t="inlineStr">
+        <is>
+          <t>12", Gate Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E190" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F190" s="60" t="n">
+        <v>11</v>
+      </c>
+      <c r="G190" s="97" t="n">
+        <v>2799</v>
+      </c>
+      <c r="H190" s="97" t="n">
+        <v>2419</v>
+      </c>
+      <c r="I190" s="97" t="n">
+        <v>4600</v>
+      </c>
       <c r="J190" s="91" t="n"/>
       <c r="K190" s="91" t="n"/>
       <c r="L190" s="92">
-        <f>IFERROR(AVERAGEIF(G190:K190,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M190" s="93" t="n"/>
-      <c r="N190" s="93" t="n"/>
-      <c r="O190" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G190:K190),"-")</f>
+        <v/>
+      </c>
+      <c r="M190" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N190" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O190" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P190" s="93" t="n"/>
       <c r="Q190" s="93" t="n"/>
       <c r="R190" s="92">
@@ -10804,7 +11261,11 @@
         <f>IFERROR(INDEX(M190:Q190,MATCH(MIN(G190:K190),G190:K190,0)),"-")</f>
         <v/>
       </c>
-      <c r="T190" t="inlineStr"/>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="191" ht="24" customHeight="1">
       <c r="A191" s="90" t="n">
@@ -10815,21 +11276,49 @@
           <t>OZEL-182</t>
         </is>
       </c>
-      <c r="D191" s="21" t="n"/>
-      <c r="E191" s="60" t="n"/>
-      <c r="F191" s="60" t="n"/>
-      <c r="G191" s="91" t="n"/>
-      <c r="H191" s="91" t="n"/>
-      <c r="I191" s="91" t="n"/>
+      <c r="D191" s="21" t="inlineStr">
+        <is>
+          <t>4", Gate Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E191" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F191" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G191" s="97" t="n">
+        <v>490.05</v>
+      </c>
+      <c r="H191" s="97" t="n">
+        <v>478</v>
+      </c>
+      <c r="I191" s="97" t="n">
+        <v>992</v>
+      </c>
       <c r="J191" s="91" t="n"/>
       <c r="K191" s="91" t="n"/>
       <c r="L191" s="92">
-        <f>IFERROR(AVERAGEIF(G191:K191,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M191" s="93" t="n"/>
-      <c r="N191" s="93" t="n"/>
-      <c r="O191" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G191:K191),"-")</f>
+        <v/>
+      </c>
+      <c r="M191" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N191" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O191" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P191" s="93" t="n"/>
       <c r="Q191" s="93" t="n"/>
       <c r="R191" s="92">
@@ -10840,7 +11329,11 @@
         <f>IFERROR(INDEX(M191:Q191,MATCH(MIN(G191:K191),G191:K191,0)),"-")</f>
         <v/>
       </c>
-      <c r="T191" t="inlineStr"/>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="192" ht="24" customHeight="1">
       <c r="A192" s="90" t="n">
@@ -10851,21 +11344,49 @@
           <t>OZEL-183</t>
         </is>
       </c>
-      <c r="D192" s="21" t="n"/>
-      <c r="E192" s="60" t="n"/>
-      <c r="F192" s="60" t="n"/>
-      <c r="G192" s="91" t="n"/>
-      <c r="H192" s="91" t="n"/>
-      <c r="I192" s="91" t="n"/>
+      <c r="D192" s="21" t="inlineStr">
+        <is>
+          <t>6", Gate Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E192" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F192" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G192" s="97" t="n">
+        <v>789.75</v>
+      </c>
+      <c r="H192" s="97" t="n">
+        <v>757</v>
+      </c>
+      <c r="I192" s="97" t="n">
+        <v>1564</v>
+      </c>
       <c r="J192" s="91" t="n"/>
       <c r="K192" s="91" t="n"/>
       <c r="L192" s="92">
-        <f>IFERROR(AVERAGEIF(G192:K192,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M192" s="93" t="n"/>
-      <c r="N192" s="93" t="n"/>
-      <c r="O192" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G192:K192),"-")</f>
+        <v/>
+      </c>
+      <c r="M192" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N192" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O192" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P192" s="93" t="n"/>
       <c r="Q192" s="93" t="n"/>
       <c r="R192" s="92">
@@ -10876,7 +11397,11 @@
         <f>IFERROR(INDEX(M192:Q192,MATCH(MIN(G192:K192),G192:K192,0)),"-")</f>
         <v/>
       </c>
-      <c r="T192" t="inlineStr"/>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="193" ht="24" customHeight="1">
       <c r="A193" s="90" t="n">
@@ -10887,21 +11412,49 @@
           <t>OZEL-184</t>
         </is>
       </c>
-      <c r="D193" s="21" t="n"/>
-      <c r="E193" s="60" t="n"/>
-      <c r="F193" s="60" t="n"/>
-      <c r="G193" s="91" t="n"/>
-      <c r="H193" s="91" t="n"/>
-      <c r="I193" s="91" t="n"/>
+      <c r="D193" s="21" t="inlineStr">
+        <is>
+          <t>8", Gate Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E193" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F193" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="G193" s="97" t="n">
+        <v>1283.85</v>
+      </c>
+      <c r="H193" s="97" t="n">
+        <v>1104</v>
+      </c>
+      <c r="I193" s="97" t="n">
+        <v>2124</v>
+      </c>
       <c r="J193" s="91" t="n"/>
       <c r="K193" s="91" t="n"/>
       <c r="L193" s="92">
-        <f>IFERROR(AVERAGEIF(G193:K193,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M193" s="93" t="n"/>
-      <c r="N193" s="93" t="n"/>
-      <c r="O193" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G193:K193),"-")</f>
+        <v/>
+      </c>
+      <c r="M193" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N193" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O193" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P193" s="93" t="n"/>
       <c r="Q193" s="93" t="n"/>
       <c r="R193" s="92">
@@ -10912,7 +11465,11 @@
         <f>IFERROR(INDEX(M193:Q193,MATCH(MIN(G193:K193),G193:K193,0)),"-")</f>
         <v/>
       </c>
-      <c r="T193" t="inlineStr"/>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="194" ht="24" customHeight="1">
       <c r="A194" s="90" t="n">
@@ -10923,21 +11480,49 @@
           <t>OZEL-185</t>
         </is>
       </c>
-      <c r="D194" s="21" t="n"/>
-      <c r="E194" s="60" t="n"/>
-      <c r="F194" s="60" t="n"/>
-      <c r="G194" s="91" t="n"/>
-      <c r="H194" s="91" t="n"/>
-      <c r="I194" s="91" t="n"/>
+      <c r="D194" s="21" t="inlineStr">
+        <is>
+          <t>4", Gate Valve, Flanged Ends, ASTM A216 WCB, 300# RF</t>
+        </is>
+      </c>
+      <c r="E194" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F194" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G194" s="97" t="n">
+        <v>575.96</v>
+      </c>
+      <c r="H194" s="97" t="n">
+        <v>745</v>
+      </c>
+      <c r="I194" s="97" t="n">
+        <v>1424</v>
+      </c>
       <c r="J194" s="91" t="n"/>
       <c r="K194" s="91" t="n"/>
       <c r="L194" s="92">
-        <f>IFERROR(AVERAGEIF(G194:K194,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M194" s="93" t="n"/>
-      <c r="N194" s="93" t="n"/>
-      <c r="O194" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G194:K194),"-")</f>
+        <v/>
+      </c>
+      <c r="M194" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N194" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O194" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P194" s="93" t="n"/>
       <c r="Q194" s="93" t="n"/>
       <c r="R194" s="92">
@@ -10948,7 +11533,11 @@
         <f>IFERROR(INDEX(M194:Q194,MATCH(MIN(G194:K194),G194:K194,0)),"-")</f>
         <v/>
       </c>
-      <c r="T194" t="inlineStr"/>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="195" ht="24" customHeight="1">
       <c r="A195" s="90" t="n">
@@ -10959,21 +11548,49 @@
           <t>OZEL-186</t>
         </is>
       </c>
-      <c r="D195" s="21" t="n"/>
-      <c r="E195" s="60" t="n"/>
-      <c r="F195" s="60" t="n"/>
-      <c r="G195" s="91" t="n"/>
-      <c r="H195" s="91" t="n"/>
-      <c r="I195" s="91" t="n"/>
+      <c r="D195" s="21" t="inlineStr">
+        <is>
+          <t>3", Swing Check Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E195" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F195" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G195" s="97" t="n">
+        <v>409.5</v>
+      </c>
+      <c r="H195" s="97" t="n">
+        <v>254</v>
+      </c>
+      <c r="I195" s="97" t="n">
+        <v>532</v>
+      </c>
       <c r="J195" s="91" t="n"/>
       <c r="K195" s="91" t="n"/>
       <c r="L195" s="92">
-        <f>IFERROR(AVERAGEIF(G195:K195,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M195" s="93" t="n"/>
-      <c r="N195" s="93" t="n"/>
-      <c r="O195" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G195:K195),"-")</f>
+        <v/>
+      </c>
+      <c r="M195" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N195" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O195" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P195" s="93" t="n"/>
       <c r="Q195" s="93" t="n"/>
       <c r="R195" s="92">
@@ -10984,7 +11601,11 @@
         <f>IFERROR(INDEX(M195:Q195,MATCH(MIN(G195:K195),G195:K195,0)),"-")</f>
         <v/>
       </c>
-      <c r="T195" t="inlineStr"/>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="196" ht="24" customHeight="1">
       <c r="A196" s="90" t="n">
@@ -10995,21 +11616,49 @@
           <t>OZEL-187</t>
         </is>
       </c>
-      <c r="D196" s="21" t="n"/>
-      <c r="E196" s="60" t="n"/>
-      <c r="F196" s="60" t="n"/>
-      <c r="G196" s="91" t="n"/>
-      <c r="H196" s="91" t="n"/>
-      <c r="I196" s="91" t="n"/>
+      <c r="D196" s="21" t="inlineStr">
+        <is>
+          <t>4", Swing Check Valve, Flanged Ends, ASTM A216 WCB, 150# RF</t>
+        </is>
+      </c>
+      <c r="E196" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F196" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G196" s="97" t="n">
+        <v>551.25</v>
+      </c>
+      <c r="H196" s="97" t="n">
+        <v>359</v>
+      </c>
+      <c r="I196" s="97" t="n">
+        <v>784</v>
+      </c>
       <c r="J196" s="91" t="n"/>
       <c r="K196" s="91" t="n"/>
       <c r="L196" s="92">
-        <f>IFERROR(AVERAGEIF(G196:K196,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M196" s="93" t="n"/>
-      <c r="N196" s="93" t="n"/>
-      <c r="O196" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G196:K196),"-")</f>
+        <v/>
+      </c>
+      <c r="M196" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N196" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O196" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P196" s="93" t="n"/>
       <c r="Q196" s="93" t="n"/>
       <c r="R196" s="92">
@@ -11020,7 +11669,11 @@
         <f>IFERROR(INDEX(M196:Q196,MATCH(MIN(G196:K196),G196:K196,0)),"-")</f>
         <v/>
       </c>
-      <c r="T196" t="inlineStr"/>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="197" ht="24" customHeight="1">
       <c r="A197" s="90" t="n">
@@ -11031,21 +11684,49 @@
           <t>OZEL-188</t>
         </is>
       </c>
-      <c r="D197" s="61" t="n"/>
-      <c r="E197" s="60" t="n"/>
-      <c r="F197" s="60" t="n"/>
-      <c r="G197" s="91" t="n"/>
-      <c r="H197" s="91" t="n"/>
-      <c r="I197" s="91" t="n"/>
+      <c r="D197" s="61" t="inlineStr">
+        <is>
+          <t>4", Swing Check Valve, Flanged Ends, ASTM A216 WCB, 300# RF</t>
+        </is>
+      </c>
+      <c r="E197" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F197" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="G197" s="97" t="n">
+        <v>610.75</v>
+      </c>
+      <c r="H197" s="97" t="n">
+        <v>466</v>
+      </c>
+      <c r="I197" s="97" t="n">
+        <v>1216</v>
+      </c>
       <c r="J197" s="91" t="n"/>
       <c r="K197" s="91" t="n"/>
       <c r="L197" s="92">
-        <f>IFERROR(AVERAGEIF(G197:K197,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M197" s="93" t="n"/>
-      <c r="N197" s="93" t="n"/>
-      <c r="O197" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G197:K197),"-")</f>
+        <v/>
+      </c>
+      <c r="M197" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N197" s="93" t="inlineStr">
+        <is>
+          <t>GELİŞİM VANA</t>
+        </is>
+      </c>
+      <c r="O197" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="P197" s="93" t="n"/>
       <c r="Q197" s="93" t="n"/>
       <c r="R197" s="92">
@@ -11056,7 +11737,11 @@
         <f>IFERROR(INDEX(M197:Q197,MATCH(MIN(G197:K197),G197:K197,0)),"-")</f>
         <v/>
       </c>
-      <c r="T197" t="inlineStr"/>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="198" ht="24" customHeight="1">
       <c r="A198" s="90" t="n">
@@ -11067,20 +11752,42 @@
           <t>OZEL-189</t>
         </is>
       </c>
-      <c r="D198" s="61" t="n"/>
-      <c r="E198" s="60" t="n"/>
-      <c r="F198" s="60" t="n"/>
-      <c r="G198" s="91" t="n"/>
-      <c r="H198" s="91" t="n"/>
+      <c r="D198" s="61" t="inlineStr">
+        <is>
+          <t>8", Butterfly Valve, Lug Type, API 609, 150# RF</t>
+        </is>
+      </c>
+      <c r="E198" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F198" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="G198" s="97" t="n">
+        <v>380</v>
+      </c>
+      <c r="H198" s="97" t="n">
+        <v>1192</v>
+      </c>
       <c r="I198" s="91" t="n"/>
       <c r="J198" s="91" t="n"/>
       <c r="K198" s="91" t="n"/>
       <c r="L198" s="92">
-        <f>IFERROR(AVERAGEIF(G198:K198,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M198" s="93" t="n"/>
-      <c r="N198" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G198:K198),"-")</f>
+        <v/>
+      </c>
+      <c r="M198" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N198" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="O198" s="93" t="n"/>
       <c r="P198" s="93" t="n"/>
       <c r="Q198" s="93" t="n"/>
@@ -11092,7 +11799,11 @@
         <f>IFERROR(INDEX(M198:Q198,MATCH(MIN(G198:K198),G198:K198,0)),"-")</f>
         <v/>
       </c>
-      <c r="T198" t="inlineStr"/>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="199" ht="24" customHeight="1">
       <c r="A199" s="90" t="n">
@@ -11103,20 +11814,42 @@
           <t>OZEL-190</t>
         </is>
       </c>
-      <c r="D199" s="61" t="n"/>
-      <c r="E199" s="60" t="n"/>
-      <c r="F199" s="60" t="n"/>
-      <c r="G199" s="91" t="n"/>
-      <c r="H199" s="91" t="n"/>
+      <c r="D199" s="61" t="inlineStr">
+        <is>
+          <t>8", Butterfly Valve, Lug Type, API 609, 150# RF</t>
+        </is>
+      </c>
+      <c r="E199" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F199" s="60" t="n">
+        <v>6</v>
+      </c>
+      <c r="G199" s="97" t="n">
+        <v>551</v>
+      </c>
+      <c r="H199" s="97" t="n">
+        <v>1192</v>
+      </c>
       <c r="I199" s="91" t="n"/>
       <c r="J199" s="91" t="n"/>
       <c r="K199" s="91" t="n"/>
       <c r="L199" s="92">
-        <f>IFERROR(AVERAGEIF(G199:K199,"&gt;0"),"-")</f>
-        <v/>
-      </c>
-      <c r="M199" s="93" t="n"/>
-      <c r="N199" s="93" t="n"/>
+        <f>IFERROR(AVERAGE(G199:K199),"-")</f>
+        <v/>
+      </c>
+      <c r="M199" s="93" t="inlineStr">
+        <is>
+          <t>EMS VANA</t>
+        </is>
+      </c>
+      <c r="N199" s="93" t="inlineStr">
+        <is>
+          <t>UNİVAL</t>
+        </is>
+      </c>
       <c r="O199" s="93" t="n"/>
       <c r="P199" s="93" t="n"/>
       <c r="Q199" s="93" t="n"/>
@@ -11128,7 +11861,11 @@
         <f>IFERROR(INDEX(M199:Q199,MATCH(MIN(G199:K199),G199:K199,0)),"-")</f>
         <v/>
       </c>
-      <c r="T199" t="inlineStr"/>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>VANA</t>
+        </is>
+      </c>
     </row>
     <row r="200" ht="24" customHeight="1">
       <c r="A200" s="90" t="n">
@@ -11148,7 +11885,7 @@
       <c r="J200" s="91" t="n"/>
       <c r="K200" s="91" t="n"/>
       <c r="L200" s="92">
-        <f>IFERROR(AVERAGEIF(G200:K200,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G200:K200),"-")</f>
         <v/>
       </c>
       <c r="M200" s="93" t="n"/>
@@ -11164,7 +11901,6 @@
         <f>IFERROR(INDEX(M200:Q200,MATCH(MIN(G200:K200),G200:K200,0)),"-")</f>
         <v/>
       </c>
-      <c r="T200" t="inlineStr"/>
     </row>
     <row r="201" ht="24" customHeight="1">
       <c r="A201" s="90" t="n">
@@ -11184,7 +11920,7 @@
       <c r="J201" s="91" t="n"/>
       <c r="K201" s="91" t="n"/>
       <c r="L201" s="92">
-        <f>IFERROR(AVERAGEIF(G201:K201,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G201:K201),"-")</f>
         <v/>
       </c>
       <c r="M201" s="93" t="n"/>
@@ -11200,7 +11936,6 @@
         <f>IFERROR(INDEX(M201:Q201,MATCH(MIN(G201:K201),G201:K201,0)),"-")</f>
         <v/>
       </c>
-      <c r="T201" t="inlineStr"/>
     </row>
     <row r="202" ht="24" customHeight="1">
       <c r="A202" s="90" t="n">
@@ -11220,7 +11955,7 @@
       <c r="J202" s="91" t="n"/>
       <c r="K202" s="91" t="n"/>
       <c r="L202" s="92">
-        <f>IFERROR(AVERAGEIF(G202:K202,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G202:K202),"-")</f>
         <v/>
       </c>
       <c r="M202" s="93" t="n"/>
@@ -11236,7 +11971,6 @@
         <f>IFERROR(INDEX(M202:Q202,MATCH(MIN(G202:K202),G202:K202,0)),"-")</f>
         <v/>
       </c>
-      <c r="T202" t="inlineStr"/>
     </row>
     <row r="203" ht="24" customHeight="1">
       <c r="A203" s="90" t="n">
@@ -11256,7 +11990,7 @@
       <c r="J203" s="91" t="n"/>
       <c r="K203" s="91" t="n"/>
       <c r="L203" s="92">
-        <f>IFERROR(AVERAGEIF(G203:K203,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G203:K203),"-")</f>
         <v/>
       </c>
       <c r="M203" s="93" t="n"/>
@@ -11272,7 +12006,6 @@
         <f>IFERROR(INDEX(M203:Q203,MATCH(MIN(G203:K203),G203:K203,0)),"-")</f>
         <v/>
       </c>
-      <c r="T203" t="inlineStr"/>
     </row>
     <row r="204" ht="24" customHeight="1">
       <c r="A204" s="90" t="n">
@@ -11292,7 +12025,7 @@
       <c r="J204" s="91" t="n"/>
       <c r="K204" s="91" t="n"/>
       <c r="L204" s="92">
-        <f>IFERROR(AVERAGEIF(G204:K204,"&gt;0"),"-")</f>
+        <f>IFERROR(AVERAGE(G204:K204),"-")</f>
         <v/>
       </c>
       <c r="M204" s="93" t="n"/>
@@ -11308,7 +12041,6 @@
         <f>IFERROR(INDEX(M204:Q204,MATCH(MIN(G204:K204),G204:K204,0)),"-")</f>
         <v/>
       </c>
-      <c r="T204" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="C9:W9">

</xml_diff>

<commit_message>
Teklif dökümantasyonu v6: ZERAY PLASTİK ve NORMTEKNİK eklendi
- ZERAY PLASTİK (TL) → HDPE boru ve fitting kalemleri (OZEL-155..165):
  DN200/300 Koruge Perforeli+Düz Boru, DN200 Te/Dirsek45/Dirsek90,
  DN25 PE100, DN50/75/110/150 Koruge Boru — net indirimli TL birim fiyatlar
- NORMTEKNİK (USD) → OZEL-191: Dış Saha Yangın Dolabı DSH-2-110 — 518,23 USD/ad
- Toplam 57 satırda fiyat verisi (önceki 45'ten 12 yeni kalem)

https://claude.ai/code/session_01Y89WpFkMWfULFiod1eBJCP
</commit_message>
<xml_diff>
--- a/TEKLIF DOKUMANTASYON.xlsx
+++ b/TEKLIF DOKUMANTASYON.xlsx
@@ -9715,7 +9715,9 @@
       </c>
       <c r="E164" s="60" t="n"/>
       <c r="F164" s="60" t="n"/>
-      <c r="G164" s="91" t="n"/>
+      <c r="G164" s="98" t="n">
+        <v>155.74</v>
+      </c>
       <c r="H164" s="91" t="n"/>
       <c r="I164" s="91" t="n"/>
       <c r="J164" s="91" t="n"/>
@@ -9724,7 +9726,11 @@
         <f>IFERROR(AVERAGE(G164:K164),"-")</f>
         <v/>
       </c>
-      <c r="M164" s="93" t="n"/>
+      <c r="M164" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N164" s="93" t="n"/>
       <c r="O164" s="93" t="n"/>
       <c r="P164" s="93" t="n"/>
@@ -9759,7 +9765,9 @@
       </c>
       <c r="E165" s="60" t="n"/>
       <c r="F165" s="60" t="n"/>
-      <c r="G165" s="91" t="n"/>
+      <c r="G165" s="98" t="n">
+        <v>145.17</v>
+      </c>
       <c r="H165" s="91" t="n"/>
       <c r="I165" s="91" t="n"/>
       <c r="J165" s="91" t="n"/>
@@ -9768,7 +9776,11 @@
         <f>IFERROR(AVERAGE(G165:K165),"-")</f>
         <v/>
       </c>
-      <c r="M165" s="93" t="n"/>
+      <c r="M165" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N165" s="93" t="n"/>
       <c r="O165" s="93" t="n"/>
       <c r="P165" s="93" t="n"/>
@@ -9803,7 +9815,9 @@
       </c>
       <c r="E166" s="60" t="n"/>
       <c r="F166" s="60" t="n"/>
-      <c r="G166" s="91" t="n"/>
+      <c r="G166" s="98" t="n">
+        <v>327.97</v>
+      </c>
       <c r="H166" s="91" t="n"/>
       <c r="I166" s="91" t="n"/>
       <c r="J166" s="91" t="n"/>
@@ -9812,7 +9826,11 @@
         <f>IFERROR(AVERAGE(G166:K166),"-")</f>
         <v/>
       </c>
-      <c r="M166" s="93" t="n"/>
+      <c r="M166" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N166" s="93" t="n"/>
       <c r="O166" s="93" t="n"/>
       <c r="P166" s="93" t="n"/>
@@ -9847,7 +9865,9 @@
       </c>
       <c r="E167" s="60" t="n"/>
       <c r="F167" s="60" t="n"/>
-      <c r="G167" s="91" t="n"/>
+      <c r="G167" s="98" t="n">
+        <v>225.7</v>
+      </c>
       <c r="H167" s="91" t="n"/>
       <c r="I167" s="91" t="n"/>
       <c r="J167" s="91" t="n"/>
@@ -9856,7 +9876,11 @@
         <f>IFERROR(AVERAGE(G167:K167),"-")</f>
         <v/>
       </c>
-      <c r="M167" s="93" t="n"/>
+      <c r="M167" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N167" s="93" t="n"/>
       <c r="O167" s="93" t="n"/>
       <c r="P167" s="93" t="n"/>
@@ -9891,7 +9915,9 @@
       </c>
       <c r="E168" s="60" t="n"/>
       <c r="F168" s="60" t="n"/>
-      <c r="G168" s="91" t="n"/>
+      <c r="G168" s="98" t="n">
+        <v>103.09</v>
+      </c>
       <c r="H168" s="91" t="n"/>
       <c r="I168" s="91" t="n"/>
       <c r="J168" s="91" t="n"/>
@@ -9900,7 +9926,11 @@
         <f>IFERROR(AVERAGE(G168:K168),"-")</f>
         <v/>
       </c>
-      <c r="M168" s="93" t="n"/>
+      <c r="M168" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N168" s="93" t="n"/>
       <c r="O168" s="93" t="n"/>
       <c r="P168" s="93" t="n"/>
@@ -9935,7 +9965,9 @@
       </c>
       <c r="E169" s="60" t="n"/>
       <c r="F169" s="60" t="n"/>
-      <c r="G169" s="91" t="n"/>
+      <c r="G169" s="98" t="n">
+        <v>132.55</v>
+      </c>
       <c r="H169" s="91" t="n"/>
       <c r="I169" s="91" t="n"/>
       <c r="J169" s="91" t="n"/>
@@ -9944,7 +9976,11 @@
         <f>IFERROR(AVERAGE(G169:K169),"-")</f>
         <v/>
       </c>
-      <c r="M169" s="93" t="n"/>
+      <c r="M169" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N169" s="93" t="n"/>
       <c r="O169" s="93" t="n"/>
       <c r="P169" s="93" t="n"/>
@@ -9979,7 +10015,9 @@
       </c>
       <c r="E170" s="60" t="n"/>
       <c r="F170" s="60" t="n"/>
-      <c r="G170" s="91" t="n"/>
+      <c r="G170" s="98" t="n">
+        <v>22.28</v>
+      </c>
       <c r="H170" s="91" t="n"/>
       <c r="I170" s="91" t="n"/>
       <c r="J170" s="91" t="n"/>
@@ -9988,7 +10026,11 @@
         <f>IFERROR(AVERAGE(G170:K170),"-")</f>
         <v/>
       </c>
-      <c r="M170" s="93" t="n"/>
+      <c r="M170" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N170" s="93" t="n"/>
       <c r="O170" s="93" t="n"/>
       <c r="P170" s="93" t="n"/>
@@ -10023,7 +10065,9 @@
       </c>
       <c r="E171" s="60" t="n"/>
       <c r="F171" s="60" t="n"/>
-      <c r="G171" s="91" t="n"/>
+      <c r="G171" s="98" t="n">
+        <v>25.2</v>
+      </c>
       <c r="H171" s="91" t="n"/>
       <c r="I171" s="91" t="n"/>
       <c r="J171" s="91" t="n"/>
@@ -10032,7 +10076,11 @@
         <f>IFERROR(AVERAGE(G171:K171),"-")</f>
         <v/>
       </c>
-      <c r="M171" s="93" t="n"/>
+      <c r="M171" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N171" s="93" t="n"/>
       <c r="O171" s="93" t="n"/>
       <c r="P171" s="93" t="n"/>
@@ -10067,7 +10115,9 @@
       </c>
       <c r="E172" s="60" t="n"/>
       <c r="F172" s="60" t="n"/>
-      <c r="G172" s="91" t="n"/>
+      <c r="G172" s="98" t="n">
+        <v>38.5</v>
+      </c>
       <c r="H172" s="91" t="n"/>
       <c r="I172" s="91" t="n"/>
       <c r="J172" s="91" t="n"/>
@@ -10076,7 +10126,11 @@
         <f>IFERROR(AVERAGE(G172:K172),"-")</f>
         <v/>
       </c>
-      <c r="M172" s="93" t="n"/>
+      <c r="M172" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N172" s="93" t="n"/>
       <c r="O172" s="93" t="n"/>
       <c r="P172" s="93" t="n"/>
@@ -10111,7 +10165,9 @@
       </c>
       <c r="E173" s="60" t="n"/>
       <c r="F173" s="60" t="n"/>
-      <c r="G173" s="91" t="n"/>
+      <c r="G173" s="98" t="n">
+        <v>47.17</v>
+      </c>
       <c r="H173" s="91" t="n"/>
       <c r="I173" s="91" t="n"/>
       <c r="J173" s="91" t="n"/>
@@ -10120,7 +10176,11 @@
         <f>IFERROR(AVERAGE(G173:K173),"-")</f>
         <v/>
       </c>
-      <c r="M173" s="93" t="n"/>
+      <c r="M173" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N173" s="93" t="n"/>
       <c r="O173" s="93" t="n"/>
       <c r="P173" s="93" t="n"/>
@@ -10155,7 +10215,9 @@
       </c>
       <c r="E174" s="60" t="n"/>
       <c r="F174" s="60" t="n"/>
-      <c r="G174" s="91" t="n"/>
+      <c r="G174" s="98" t="n">
+        <v>92.37</v>
+      </c>
       <c r="H174" s="91" t="n"/>
       <c r="I174" s="91" t="n"/>
       <c r="J174" s="91" t="n"/>
@@ -10164,7 +10226,11 @@
         <f>IFERROR(AVERAGE(G174:K174),"-")</f>
         <v/>
       </c>
-      <c r="M174" s="93" t="n"/>
+      <c r="M174" s="93" t="inlineStr">
+        <is>
+          <t>ZERAY PLASTİK</t>
+        </is>
+      </c>
       <c r="N174" s="93" t="n"/>
       <c r="O174" s="93" t="n"/>
       <c r="P174" s="93" t="n"/>
@@ -11876,10 +11942,22 @@
           <t>OZEL-191</t>
         </is>
       </c>
-      <c r="D200" s="61" t="n"/>
-      <c r="E200" s="60" t="n"/>
-      <c r="F200" s="60" t="n"/>
-      <c r="G200" s="91" t="n"/>
+      <c r="D200" s="61" t="inlineStr">
+        <is>
+          <t>Dış Saha Yangın Dolabı DSH-2-110, 700x1100x200, 2x2½" Hortum, RAL3001</t>
+        </is>
+      </c>
+      <c r="E200" s="60" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+      <c r="F200" s="60" t="n">
+        <v>13</v>
+      </c>
+      <c r="G200" s="97" t="n">
+        <v>518.23</v>
+      </c>
       <c r="H200" s="91" t="n"/>
       <c r="I200" s="91" t="n"/>
       <c r="J200" s="91" t="n"/>
@@ -11888,7 +11966,11 @@
         <f>IFERROR(AVERAGE(G200:K200),"-")</f>
         <v/>
       </c>
-      <c r="M200" s="93" t="n"/>
+      <c r="M200" s="93" t="inlineStr">
+        <is>
+          <t>NORMTEKNİK</t>
+        </is>
+      </c>
       <c r="N200" s="93" t="n"/>
       <c r="O200" s="93" t="n"/>
       <c r="P200" s="93" t="n"/>

</xml_diff>